<commit_message>
docs: link both UI pull requests in the council workbook
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -22,7 +22,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
@@ -163,7 +163,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deferred</t>
+          <t xml:space="preserve">Pending advisory</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -8501,10 +8501,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="65" customWidth="1"/>
+    <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8551,8 +8551,30 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Busnes-app/KyNotes-server</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/Busnes-app/KyNotes-server/pull/118</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/notes-eight</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Editor, phone navigation and frozen council evidence; no merge/deployment</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: audit Gemini advice and retain its raw scores
Preserve the original Argon reports with their inconsistent weights and factual claims. Record source and native-browser evidence rejecting the missing desktop rail and inaccessible footer claims, and defer valid optional polish. Include raw and fixed-rubric calculations without treating the advisory rating as progression evidence.
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -22,7 +22,7 @@
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="70" customWidth="1"/>
   </cols>
@@ -101,7 +101,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separate raw verdicts; see each original review for cohort means and limits.</t>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
         </is>
       </c>
     </row>
@@ -137,7 +137,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separate raw verdicts; see each original review for cohort means and limits.</t>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
         </is>
       </c>
     </row>
@@ -163,17 +163,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pending advisory</t>
+          <t xml:space="preserve">8.1/10 (raw*)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">True</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separate raw verdicts; see each original review for cohort means and limits.</t>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
         </is>
       </c>
     </row>
@@ -195,11 +195,12 @@
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="21" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="13" width="59" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="70" customWidth="1"/>
+    <col min="16" max="16" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -255,12 +256,12 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Computed quality</t>
+          <t xml:space="preserve">Fixed-rubric quality</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reported quality</t>
+          <t xml:space="preserve">Raw reported quality</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -276,6 +277,11 @@
       <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">Caveat</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declared weights conform</t>
         </is>
       </c>
     </row>
@@ -332,6 +338,11 @@
           <t xml:space="preserve">Fixture paragraph spacing (typed blank line) and trailing empty bullet inflate the H2 gap; cannot show hover, focus or scroll behaviour.</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -386,6 +397,11 @@
           <t xml:space="preserve">Near-duplicate of after-workspace-mobile (0.0036-0.0046% px, max delta 4); cannot show focus return or scrolling.</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -440,6 +456,11 @@
           <t xml:space="preserve">Synthetic account always shows the recovery callout; real accounts with a saved recovery code would see rows earlier. Rows are reachable by inner scroll (Playwright auto-scrolls), which the image cannot show.</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -494,6 +515,11 @@
           <t xml:space="preserve">Unmatched to before: after shows 'Research notes' open (test selected it), before shows 'Launch checklist'.</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -548,6 +574,11 @@
           <t xml:space="preserve">Byte-identical to before; unchanged by this diff.</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -602,6 +633,11 @@
           <t xml:space="preserve">Byte-identical to before; unchanged by this diff.</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -656,6 +692,11 @@
           <t xml:space="preserve">Fixture paragraph spacing (typed blank line) and trailing empty bullet inflate the H2 gap; cannot show hover, focus or scroll behaviour.</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -710,6 +751,11 @@
           <t xml:space="preserve">Near-duplicate of after-workspace-mobile (0.0036-0.0046% px, max delta 4); cannot show focus return or scrolling.</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -764,6 +810,11 @@
           <t xml:space="preserve">Synthetic account always shows the recovery callout; real accounts with a saved recovery code would see rows earlier. Rows are reachable by inner scroll (Playwright auto-scrolls), which the image cannot show.</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -818,6 +869,11 @@
           <t xml:space="preserve">Unmatched to before: after shows 'Research notes' open (test selected it), before shows 'Launch checklist'.</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -872,6 +928,11 @@
           <t xml:space="preserve">Byte-identical to before; unchanged by this diff.</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -926,6 +987,11 @@
           <t xml:space="preserve">Byte-identical to before; unchanged by this diff.</t>
         </is>
       </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -980,6 +1046,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1034,6 +1105,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1088,6 +1164,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1142,6 +1223,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1196,6 +1282,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1250,6 +1341,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1304,6 +1400,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1358,6 +1459,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1412,6 +1518,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1466,6 +1577,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1520,6 +1636,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1574,6 +1695,11 @@
           <t xml:space="preserve">Static 1x capture: no hover, focus, loading, error or named-theme states; light and dark scored identically because no theme-specific defect is visible.</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1628,6 +1754,11 @@
           <t xml:space="preserve">Populated 4-page fixture; editor scrolls past the fold so Comments and attachments are only partly visible. workspace-desktop-light is a near duplicate.</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1682,6 +1813,11 @@
           <t xml:space="preserve">Populated 4-page fixture; editor scrolls past the fold so Comments and attachments are only partly visible. workspace-desktop-dark is a near duplicate.</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1736,6 +1872,11 @@
           <t xml:space="preserve">Editor below the fold (Outdent, Delete, Comments) not visible. workspace-mobile-light is a near duplicate.</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1790,6 +1931,11 @@
           <t xml:space="preserve">Editor below the fold (Outdent, Delete, Comments) not visible. workspace-mobile-dark is a near duplicate.</t>
         </is>
       </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1844,6 +1990,11 @@
           <t xml:space="preserve">Sparse state (4 pages); fixture previews are identical text, so preview variety is not shown.</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1898,6 +2049,11 @@
           <t xml:space="preserve">Sparse state (4 pages); fixture previews are identical text, so preview variety is not shown.</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1952,6 +2108,11 @@
           <t xml:space="preserve">Captured with 'Research notes' open, a different page from the editor capture; fixture order, not a defect.</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2006,6 +2167,11 @@
           <t xml:space="preserve">Captured with 'Research notes' open, a different page from the editor capture; fixture order, not a defect.</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2060,6 +2226,11 @@
           <t xml:space="preserve">Grid continues below the fold; Reminders/Password/devices sections not captured.</t>
         </is>
       </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2114,6 +2285,11 @@
           <t xml:space="preserve">Grid continues below the fold; Reminders/Password/devices sections not captured.</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2168,6 +2344,11 @@
           <t xml:space="preserve">Only two card rows visible; remaining catalog and sections below the fold.</t>
         </is>
       </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2222,6 +2403,11 @@
           <t xml:space="preserve">Only two card rows visible; remaining catalog and sections below the fold.</t>
         </is>
       </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2276,6 +2462,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2330,6 +2521,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2384,6 +2580,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2438,6 +2639,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2492,6 +2698,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2546,6 +2757,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2600,6 +2816,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2654,6 +2875,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2708,6 +2934,11 @@
           <t xml:space="preserve">Expanded notebook-navigation comparison is unmatched: after has Research notes selected, before Launch checklist; account initials also differ between fresh fixtures.</t>
         </is>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2762,6 +2993,11 @@
           <t xml:space="preserve">Expanded notebook-navigation comparison is unmatched: after has Research notes selected, before Launch checklist; account initials also differ between fresh fixtures.</t>
         </is>
       </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2816,6 +3052,11 @@
           <t xml:space="preserve">The open page pane has its own scroller; screenshots show neither its hidden rows nor their behavior.</t>
         </is>
       </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2870,6 +3111,11 @@
           <t xml:space="preserve">The open page pane has its own scroller; screenshots show neither its hidden rows nor their behavior.</t>
         </is>
       </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2929,6 +3175,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2988,6 +3239,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3047,6 +3303,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3106,6 +3367,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3165,6 +3431,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3224,6 +3495,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3283,6 +3559,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3342,6 +3623,11 @@
           <t xml:space="preserve">Only the first part of the theme catalog is visible; no theme selection or all-theme contrast is proven.</t>
         </is>
       </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3396,6 +3682,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3450,6 +3741,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3504,6 +3800,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3558,6 +3859,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3612,6 +3918,11 @@
           <t xml:space="preserve">Expanded notebook-navigation comparison is unmatched: after has Research notes selected, before Launch checklist; account initials also differ between fresh fixtures.</t>
         </is>
       </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3666,6 +3977,11 @@
           <t xml:space="preserve">Expanded notebook-navigation comparison is unmatched: after has Research notes selected, before Launch checklist; account initials also differ between fresh fixtures.</t>
         </is>
       </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3725,6 +4041,11 @@
           <t xml:space="preserve">The open page pane has its own scroller; screenshots show neither its hidden rows nor their behavior.</t>
         </is>
       </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3784,6 +4105,11 @@
           <t xml:space="preserve">The open page pane has its own scroller; screenshots show neither its hidden rows nor their behavior.</t>
         </is>
       </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3843,6 +4169,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3902,6 +4233,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3961,6 +4297,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4020,6 +4361,11 @@
           <t xml:space="preserve">Synthetic four-page fixture with a trailing blank bullet; capture alone does not prove saving, scrolling or persisted coordinate preservation.</t>
         </is>
       </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4074,6 +4420,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Only the top of the catalog is captured; 22 named choices plus Match system are known from source, not all visible here.</t>
         </is>
       </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4128,6 +4479,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Only the top of the catalog is captured; 22 named choices plus Match system are known from source, not all visible here.</t>
         </is>
       </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4182,6 +4538,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Only the top of the catalog is captured; 22 named choices plus Match system are known from source, not all visible here.</t>
         </is>
       </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4236,6 +4597,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Only the top of the catalog is captured; 22 named choices plus Match system are known from source, not all visible here.</t>
         </is>
       </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4290,6 +4656,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Blank paragraph spacing and the trailing empty bullet belong to the synthetic document, not a product defect. Footer continuation at the phone fold is not evidence of inaccessible controls.</t>
         </is>
       </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4344,6 +4715,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Blank paragraph spacing and the trailing empty bullet belong to the synthetic document, not a product defect. Footer continuation at the phone fold is not evidence of inaccessible controls.</t>
         </is>
       </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4398,6 +4774,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Blank paragraph spacing and the trailing empty bullet belong to the synthetic document, not a product defect. Footer continuation at the phone fold is not evidence of inaccessible controls.</t>
         </is>
       </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4452,6 +4833,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Blank paragraph spacing and the trailing empty bullet belong to the synthetic document, not a product defect. Footer continuation at the phone fold is not evidence of inaccessible controls.</t>
         </is>
       </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4506,6 +4892,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Research notes is open, matching stage-02-after navigation; the original before navigation had Launch checklist and is unmatched.</t>
         </is>
       </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4560,6 +4951,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. Research notes is open, matching stage-02-after navigation; the original before navigation had Launch checklist and is unmatched.</t>
         </is>
       </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4614,6 +5010,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. The fourth selected row reaches the fold; ordinary document scrolling is needed for its full preview. Accounts with recovery configured would have a shorter preamble.</t>
         </is>
       </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4668,6 +5069,11 @@
           <t xml:space="preserve">Static populated Chromium 156 capture cannot establish keyboard, focus, contrast ratios, save preservation or other themes/states. The fourth selected row reaches the fold; ordinary document scrolling is needed for its full preview. Accounts with recovery configured would have a shorter preamble.</t>
         </is>
       </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4727,6 +5133,11 @@
           <t xml:space="preserve">Measured near duplicate of the first filename in this group; inherits that image score and observations.</t>
         </is>
       </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4786,6 +5197,11 @@
           <t xml:space="preserve">Measured near duplicate of the first filename in this group; inherits that image score and observations.</t>
         </is>
       </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4845,6 +5261,11 @@
           <t xml:space="preserve">Measured near duplicate of the first filename in this group; inherits that image score and observations.</t>
         </is>
       </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4904,6 +5325,11 @@
           <t xml:space="preserve">Measured near duplicate of the first filename in this group; inherits that image score and observations.</t>
         </is>
       </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4958,6 +5384,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5012,6 +5443,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5066,6 +5502,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5120,6 +5561,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5174,6 +5620,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5228,6 +5679,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5282,6 +5738,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5336,6 +5797,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5390,6 +5856,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5444,6 +5915,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5498,6 +5974,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5552,6 +6033,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. Navigation state and content count are judged as captured; no extra fixture data is required.</t>
         </is>
       </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5611,6 +6097,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5670,6 +6161,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5729,6 +6225,11 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5788,9 +6289,722 @@
           <t xml:space="preserve">Static populated Chromium 156 scale-1 capture cannot prove saves, keyboard/focus, computed contrast or missing themes/states. The trailing empty bullet is intentional fixture content.</t>
         </is>
       </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E102">
+        <v>8</v>
+      </c>
+      <c r="F102">
+        <v>8</v>
+      </c>
+      <c r="G102">
+        <v>8</v>
+      </c>
+      <c r="H102">
+        <v>9</v>
+      </c>
+      <c r="I102">
+        <v>8</v>
+      </c>
+      <c r="J102">
+        <v>7</v>
+      </c>
+      <c r="K102">
+        <v>8.0</v>
+      </c>
+      <c r="L102">
+        <v>8.1</v>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E103">
+        <v>8</v>
+      </c>
+      <c r="F103">
+        <v>8</v>
+      </c>
+      <c r="G103">
+        <v>8</v>
+      </c>
+      <c r="H103">
+        <v>9</v>
+      </c>
+      <c r="I103">
+        <v>8</v>
+      </c>
+      <c r="J103">
+        <v>7</v>
+      </c>
+      <c r="K103">
+        <v>8.0</v>
+      </c>
+      <c r="L103">
+        <v>8.1</v>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E104">
+        <v>8</v>
+      </c>
+      <c r="F104">
+        <v>8</v>
+      </c>
+      <c r="G104">
+        <v>7</v>
+      </c>
+      <c r="H104">
+        <v>9</v>
+      </c>
+      <c r="I104">
+        <v>8</v>
+      </c>
+      <c r="J104">
+        <v>8</v>
+      </c>
+      <c r="K104">
+        <v>8.0</v>
+      </c>
+      <c r="L104">
+        <v>8.0</v>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B105">
+        <v>3</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E105">
+        <v>8</v>
+      </c>
+      <c r="F105">
+        <v>8</v>
+      </c>
+      <c r="G105">
+        <v>7</v>
+      </c>
+      <c r="H105">
+        <v>9</v>
+      </c>
+      <c r="I105">
+        <v>8</v>
+      </c>
+      <c r="J105">
+        <v>8</v>
+      </c>
+      <c r="K105">
+        <v>8.0</v>
+      </c>
+      <c r="L105">
+        <v>8.0</v>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B106">
+        <v>3</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E106">
+        <v>8</v>
+      </c>
+      <c r="F106">
+        <v>8</v>
+      </c>
+      <c r="G106">
+        <v>8</v>
+      </c>
+      <c r="H106">
+        <v>9</v>
+      </c>
+      <c r="I106">
+        <v>8</v>
+      </c>
+      <c r="J106">
+        <v>8</v>
+      </c>
+      <c r="K106">
+        <v>8.2</v>
+      </c>
+      <c r="L106">
+        <v>8.2</v>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B107">
+        <v>3</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E107">
+        <v>8</v>
+      </c>
+      <c r="F107">
+        <v>8</v>
+      </c>
+      <c r="G107">
+        <v>8</v>
+      </c>
+      <c r="H107">
+        <v>9</v>
+      </c>
+      <c r="I107">
+        <v>8</v>
+      </c>
+      <c r="J107">
+        <v>8</v>
+      </c>
+      <c r="K107">
+        <v>8.2</v>
+      </c>
+      <c r="L107">
+        <v>8.2</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B108">
+        <v>3</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E108">
+        <v>8</v>
+      </c>
+      <c r="F108">
+        <v>8</v>
+      </c>
+      <c r="G108">
+        <v>7</v>
+      </c>
+      <c r="H108">
+        <v>9</v>
+      </c>
+      <c r="I108">
+        <v>8</v>
+      </c>
+      <c r="J108">
+        <v>8</v>
+      </c>
+      <c r="K108">
+        <v>8.0</v>
+      </c>
+      <c r="L108">
+        <v>8.0</v>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B109">
+        <v>3</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">notes</t>
+        </is>
+      </c>
+      <c r="E109">
+        <v>8</v>
+      </c>
+      <c r="F109">
+        <v>8</v>
+      </c>
+      <c r="G109">
+        <v>7</v>
+      </c>
+      <c r="H109">
+        <v>9</v>
+      </c>
+      <c r="I109">
+        <v>8</v>
+      </c>
+      <c r="J109">
+        <v>8</v>
+      </c>
+      <c r="K109">
+        <v>8.0</v>
+      </c>
+      <c r="L109">
+        <v>8.0</v>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B110">
+        <v>3</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">settings</t>
+        </is>
+      </c>
+      <c r="E110">
+        <v>8</v>
+      </c>
+      <c r="F110">
+        <v>9</v>
+      </c>
+      <c r="G110">
+        <v>8</v>
+      </c>
+      <c r="H110">
+        <v>9</v>
+      </c>
+      <c r="I110">
+        <v>9</v>
+      </c>
+      <c r="J110">
+        <v>9</v>
+      </c>
+      <c r="K110">
+        <v>8.6</v>
+      </c>
+      <c r="L110">
+        <v>8.6</v>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B111">
+        <v>3</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">settings</t>
+        </is>
+      </c>
+      <c r="E111">
+        <v>8</v>
+      </c>
+      <c r="F111">
+        <v>9</v>
+      </c>
+      <c r="G111">
+        <v>8</v>
+      </c>
+      <c r="H111">
+        <v>9</v>
+      </c>
+      <c r="I111">
+        <v>9</v>
+      </c>
+      <c r="J111">
+        <v>9</v>
+      </c>
+      <c r="K111">
+        <v>8.6</v>
+      </c>
+      <c r="L111">
+        <v>8.6</v>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B112">
+        <v>3</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">settings</t>
+        </is>
+      </c>
+      <c r="E112">
+        <v>8</v>
+      </c>
+      <c r="F112">
+        <v>9</v>
+      </c>
+      <c r="G112">
+        <v>8</v>
+      </c>
+      <c r="H112">
+        <v>9</v>
+      </c>
+      <c r="I112">
+        <v>8</v>
+      </c>
+      <c r="J112">
+        <v>8</v>
+      </c>
+      <c r="K112">
+        <v>8.3</v>
+      </c>
+      <c r="L112">
+        <v>8.3</v>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gemini</t>
+        </is>
+      </c>
+      <c r="B113">
+        <v>3</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">settings</t>
+        </is>
+      </c>
+      <c r="E113">
+        <v>8</v>
+      </c>
+      <c r="F113">
+        <v>9</v>
+      </c>
+      <c r="G113">
+        <v>8</v>
+      </c>
+      <c r="H113">
+        <v>9</v>
+      </c>
+      <c r="I113">
+        <v>8</v>
+      </c>
+      <c r="J113">
+        <v>8</v>
+      </c>
+      <c r="K113">
+        <v>8.3</v>
+      </c>
+      <c r="L113">
+        <v>8.3</v>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">high</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scored blind from Stage-04 PNG and verified against live DOM at http://127.0.0.1:18101.</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O101"/>
+  <autoFilter ref="A1:P113"/>
 </worksheet>
 </file>
 
@@ -8058,7 +9272,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="2" max="2" width="37" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8385,8 +9599,25 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini advisory audit</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">completed; raw rating nonconforming</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Raw8.1/satisfied preserved. Ten findings audited with source and native-browser evidence; false desktop-rail and inaccessible-footer claims rejected. Valid optional polish deferred. No product source changed; prior implementation checks remain applicable.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C19"/>
+  <autoFilter ref="A1:C20"/>
 </worksheet>
 </file>
 
@@ -8477,7 +9708,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deferred until Opus and Sol satisfied; audit findings, retain raw score and rejection reasons</t>
+          <t xml:space="preserve">Raw advisory8.1 retained; nonconforming weights and unsupported facts audited. Opus/Sol determine progression; see Gemini audit.</t>
         </is>
       </c>
     </row>
@@ -8581,10 +9812,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="1" max="1" width="41" customWidth="1"/>
+    <col min="2" max="2" width="65" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8609,7 +9840,227 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G1-rubric-and-score-integrity</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rejected as comparable rating</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">argon-round3.json weights hierarchy=.25/coherence=.10; fixed ky-suite-v2=.20/.15. JSON Settings8.5; Markdown/final summary8.4. Desktop editor raw JSON8.1 vs Markdown8.0.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preserve raw Notes8.1/satisfied=true, but exclude Gemini from the progression decision. Its vectors recomputed with the fixed rubric yield Notes8.1 and Settings8.5; these calculations are not a fresh validated visual review. All12raw JSON totals match its declared weights under Decimal half-up; Markdown uses inconsistent rounding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G2-desktop-selected-rail</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rejected</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web/src/ky-ui/navigation.css selected [class].ky-nav-item rules; main.tsx selected notebook has ky-nav-item and aria-current=page. Native T3 at1280x900: Project Atlas box-shadow rgb(191,63,24) 3px 0px 0px 0px inset.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The shared base selector already supplies the desktop rail. Gemini inspected the phone override without accounting for imported shared CSS. No duplicate product rule added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G3-light-avatar-chip</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">supported; deferred optional polish</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">styles.css avatar uses panel-hover. Native light: avatar and sidebar rgb(242,239,231); avatar text rgb(86,100,97). Opus already records this.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The chip has little separation; the visible initial remains legible. Equal colors have1:1 contrast, not the claimed0:1. This is a minor coherence observation, with no blocked workflow or progression objection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G4-secondary-button-border</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">partly supported; deferred optional polish</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">styles.css secondary border uses line-strong; native Save border rgba(24,35,38,.38), label rgb(24,35,38). Strong labels and existing focus treatment identify controls.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The subtle border is real. A low border ratio alone does not prove WCAG1.4.11 failure when the control is identified by its readable label. Gemini also substitutes .38 for the dark token actual .42. Do not reopen this accepted visual pass on an unproven compliance claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G5-mobile-footer-clipping</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rejected as inaccessible clipping; density retained as optional</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Native390x844: actions second row y831.5–871.5, page scrollHeight1130. After scrolling the same page286px: Outdent/Delete y545.5–585.5, fully inside viewport.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The controls continue below the initial fold on a scrollable page. They are not horizontally clipped or unreachable. Compaction may improve density but is not a required fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G6-title-search-chevron-settings-polish</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">supported; deferred</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source and stage04 captures show24px notebook/page titles,150px desktop search, native recovery summary marker, and wrapped phone Settings links. Opus/Sol already retain these polish limits.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">These are optional refinements after the scoped8gate. The suggested --ky-text-section token and ChevronIcon in App.tsx do not exist here; actual primitives are --ky-type-section and NavIcon in NavIcon.tsx. No product change made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G7-appearance-and-status-implementation</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rejected factual descriptions</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">main.tsx Appearance is a fieldset.ky-appearance with native inputs; no ky-appearance custom element or shadow DOM. Current status is sync-dot; there is no claimed status-banner.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini describes implementation structures absent from this product. Its findings do not justify corresponding code changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G8-capture-content-and-sequence</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rejected inaccurate details</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Current four pages are Research notes, Team handover, Next steps, Launch checklist; chooser native row bounds355–636. ui-council.e2e.ts captures workspace before editor.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemini invents Project Atlas overview/Weekly review, reverses the capture order and gives mismatched coordinates. Inventory hashes stay valid, but its detailed visual observations are not fully reliable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G9-behavior-gate-claims</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">narrowed to recorded scope</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">checks.json and primary reports retain partial focus/responsive coverage; keyboard disclosure and page-selection regressions passed, full state/theme/browser matrix untested.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source inspection and a few interactions cannot certify complete keyboard/focus/responsive acceptance. Retain the actual scoped checks and full9limitations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G10-report-provenance</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rejected timestamp; raw artifact retained</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">argon-round3.json generated_at2026-04-13T21:48:00Z predates this2026-10-26 capture set. Raw model label omits the high variant; orchestration selected gemini-4-argon-high via antigravity.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use orchestration identity and capture manifests for provenance. Preserve the inaccurate original field with this correction; do not silently rewrite it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:D11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
navigation: use one left pane for notebooks and pages
Switch notebook management and page navigation within the same 240px region. Preserve management during background loads, restore focus immediately after explicit choices and retain phone/save/recovery behavior. Record the owner's rejection and fresh capture provenance, with current Council review pending.
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -25,6 +25,7 @@
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="70" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -68,6 +69,11 @@
           <t xml:space="preserve">Basis</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -104,6 +110,11 @@
           <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -140,6 +151,11 @@
           <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -176,9 +192,59 @@
           <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/10 — rejected double left navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deferred</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:I5"/>
 </worksheet>
 </file>
 
@@ -8765,8 +8831,1586 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7ddd736539fee331b093308c0dd1ff4c85e8476fc5a9be29c3b24476bb791f4c</t>
+        </is>
+      </c>
+      <c r="C66">
+        <v>70014</v>
+      </c>
+      <c r="D66">
+        <v>1280</v>
+      </c>
+      <c r="E66">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9e8b869d90fb1dbb3d61bc5165794e4c0d50d7003d3607378e091755b050f704</t>
+        </is>
+      </c>
+      <c r="C67">
+        <v>69039</v>
+      </c>
+      <c r="D67">
+        <v>1280</v>
+      </c>
+      <c r="E67">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72b2894e5a5204a913f362c7be193442de97ece5db425a294540f17c18cf7520</t>
+        </is>
+      </c>
+      <c r="C68">
+        <v>41587</v>
+      </c>
+      <c r="D68">
+        <v>390</v>
+      </c>
+      <c r="E68">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a48727c6f46ce1f3c40512a14cfaab32aa9233280c3d8ace4c42901f8fc54eab</t>
+        </is>
+      </c>
+      <c r="C69">
+        <v>41014</v>
+      </c>
+      <c r="D69">
+        <v>390</v>
+      </c>
+      <c r="E69">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">abb8b87e11114d2e7b8a7e0d094d79cc4ae38475737d19e9ee43a076edce63eb</t>
+        </is>
+      </c>
+      <c r="C70">
+        <v>79727</v>
+      </c>
+      <c r="D70">
+        <v>1280</v>
+      </c>
+      <c r="E70">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">636850b73dadbb684d3b31b7614c17a4acdc0bc53f77ba48a44dad0f08afee3b</t>
+        </is>
+      </c>
+      <c r="C71">
+        <v>78936</v>
+      </c>
+      <c r="D71">
+        <v>1280</v>
+      </c>
+      <c r="E71">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8c71a1cc4942d47450585d3bbc90108815563297a094032f90279893373e7e61</t>
+        </is>
+      </c>
+      <c r="C72">
+        <v>41995</v>
+      </c>
+      <c r="D72">
+        <v>390</v>
+      </c>
+      <c r="E72">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e7df73214f0e6fef0df1f0e3a57d768e91700060df8dcfaf0c0b98a8d90ae7dd</t>
+        </is>
+      </c>
+      <c r="C73">
+        <v>41261</v>
+      </c>
+      <c r="D73">
+        <v>390</v>
+      </c>
+      <c r="E73">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">523fd79e8946c26bc4a59fac57a92eb8d28ce66d21639703ee326fda4e9d9190</t>
+        </is>
+      </c>
+      <c r="C74">
+        <v>31841</v>
+      </c>
+      <c r="D74">
+        <v>1280</v>
+      </c>
+      <c r="E74">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8837f9997b6800ec556339037a6b17f9a3345b59b0e0ee89f6b3891e840b1d93</t>
+        </is>
+      </c>
+      <c r="C75">
+        <v>31656</v>
+      </c>
+      <c r="D75">
+        <v>1280</v>
+      </c>
+      <c r="E75">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c0a4e4a486d97a1110d9389a2e7431e168029b9c052c0a4eb43d8fa5c4426a9d</t>
+        </is>
+      </c>
+      <c r="C76">
+        <v>26174</v>
+      </c>
+      <c r="D76">
+        <v>390</v>
+      </c>
+      <c r="E76">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eff88854444211d4122afd5dbd41a0a7a0fe67d6ce77a31d1c8830a9d9763f87</t>
+        </is>
+      </c>
+      <c r="C77">
+        <v>25577</v>
+      </c>
+      <c r="D77">
+        <v>390</v>
+      </c>
+      <c r="E77">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">660f457322bfeaca470632ba6ef486aeeba43ea22e21c29ada32615d7de59a2f</t>
+        </is>
+      </c>
+      <c r="C78">
+        <v>71332</v>
+      </c>
+      <c r="D78">
+        <v>1280</v>
+      </c>
+      <c r="E78">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09aaa8a16c2e6de9308f1bee239d036a344bfac07f5b3b4045ab4577cbe0902c</t>
+        </is>
+      </c>
+      <c r="C79">
+        <v>70180</v>
+      </c>
+      <c r="D79">
+        <v>1280</v>
+      </c>
+      <c r="E79">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4386905eae64c0f5e2b235d07e0c82ab6634c6a9152f5b166153661726f442a7</t>
+        </is>
+      </c>
+      <c r="C80">
+        <v>35933</v>
+      </c>
+      <c r="D80">
+        <v>390</v>
+      </c>
+      <c r="E80">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cb25ccff9a7d0fb4111f103e434b7a560e5aaf00e3d413095268dd2164365c5d</t>
+        </is>
+      </c>
+      <c r="C81">
+        <v>34830</v>
+      </c>
+      <c r="D81">
+        <v>390</v>
+      </c>
+      <c r="E81">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34e628e3ffaa2f7f0d7de149e187185c15818fe9ae67b96c928093f186de5fef</t>
+        </is>
+      </c>
+      <c r="C82">
+        <v>35402</v>
+      </c>
+      <c r="D82">
+        <v>390</v>
+      </c>
+      <c r="E82">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bef7ce282a47256d80c1d2b28cdd2ef3d6111ad032d2d11e4bab46539525aec</t>
+        </is>
+      </c>
+      <c r="C83">
+        <v>34434</v>
+      </c>
+      <c r="D83">
+        <v>390</v>
+      </c>
+      <c r="E83">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c121214a77c2935d02a1152a30038f9da1bd6582b44bc655e0e0315560010c87</t>
+        </is>
+      </c>
+      <c r="C84">
+        <v>79729</v>
+      </c>
+      <c r="D84">
+        <v>1280</v>
+      </c>
+      <c r="E84">
+        <v>900</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H84">
+        <v>15</v>
+      </c>
+      <c r="I84">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fb0d176c282cb503526811a31a1507bd09b14d34f85dc1130b7b5f95be9ce43d</t>
+        </is>
+      </c>
+      <c r="C85">
+        <v>78931</v>
+      </c>
+      <c r="D85">
+        <v>1280</v>
+      </c>
+      <c r="E85">
+        <v>900</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H85">
+        <v>12</v>
+      </c>
+      <c r="I85">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30bd84772a120fefe3b5a34bb7d56054ecaf85fc066c52d577ef6024e00532e4</t>
+        </is>
+      </c>
+      <c r="C86">
+        <v>41996</v>
+      </c>
+      <c r="D86">
+        <v>390</v>
+      </c>
+      <c r="E86">
+        <v>844</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H86">
+        <v>15</v>
+      </c>
+      <c r="I86">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9dbeeec004801353f47f9e45520c7c129aa93bc3881e4855909609be33156cfc</t>
+        </is>
+      </c>
+      <c r="C87">
+        <v>41254</v>
+      </c>
+      <c r="D87">
+        <v>390</v>
+      </c>
+      <c r="E87">
+        <v>844</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H87">
+        <v>12</v>
+      </c>
+      <c r="I87">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7ddd736539fee331b093308c0dd1ff4c85e8476fc5a9be29c3b24476bb791f4c</t>
+        </is>
+      </c>
+      <c r="C88">
+        <v>70014</v>
+      </c>
+      <c r="D88">
+        <v>1280</v>
+      </c>
+      <c r="E88">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9e8b869d90fb1dbb3d61bc5165794e4c0d50d7003d3607378e091755b050f704</t>
+        </is>
+      </c>
+      <c r="C89">
+        <v>69039</v>
+      </c>
+      <c r="D89">
+        <v>1280</v>
+      </c>
+      <c r="E89">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72b2894e5a5204a913f362c7be193442de97ece5db425a294540f17c18cf7520</t>
+        </is>
+      </c>
+      <c r="C90">
+        <v>41587</v>
+      </c>
+      <c r="D90">
+        <v>390</v>
+      </c>
+      <c r="E90">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a48727c6f46ce1f3c40512a14cfaab32aa9233280c3d8ace4c42901f8fc54eab</t>
+        </is>
+      </c>
+      <c r="C91">
+        <v>41014</v>
+      </c>
+      <c r="D91">
+        <v>390</v>
+      </c>
+      <c r="E91">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d710fd517093bf43b1f5952b15e5b882e9f66c6178fd5b378e7bd1e5cab8f1f3</t>
+        </is>
+      </c>
+      <c r="C92">
+        <v>79652</v>
+      </c>
+      <c r="D92">
+        <v>1280</v>
+      </c>
+      <c r="E92">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dff310f13e7b07e3f0f3a70bcff14d3d4db31125f3f3b80fb1e0b7e56b0526df</t>
+        </is>
+      </c>
+      <c r="C93">
+        <v>79032</v>
+      </c>
+      <c r="D93">
+        <v>1280</v>
+      </c>
+      <c r="E93">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a33657e7fe1a45d046a05009a9cb53b8dcf6d1ee1ecc40011735dcb2a17a8976</t>
+        </is>
+      </c>
+      <c r="C94">
+        <v>41766</v>
+      </c>
+      <c r="D94">
+        <v>390</v>
+      </c>
+      <c r="E94">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d17eddc8a6bbc12345f7a39df8b00f5b0ebb18d8ee693b4c3c6dd889ea2dc7c1</t>
+        </is>
+      </c>
+      <c r="C95">
+        <v>41299</v>
+      </c>
+      <c r="D95">
+        <v>390</v>
+      </c>
+      <c r="E95">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">523fd79e8946c26bc4a59fac57a92eb8d28ce66d21639703ee326fda4e9d9190</t>
+        </is>
+      </c>
+      <c r="C96">
+        <v>31841</v>
+      </c>
+      <c r="D96">
+        <v>1280</v>
+      </c>
+      <c r="E96">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8837f9997b6800ec556339037a6b17f9a3345b59b0e0ee89f6b3891e840b1d93</t>
+        </is>
+      </c>
+      <c r="C97">
+        <v>31656</v>
+      </c>
+      <c r="D97">
+        <v>1280</v>
+      </c>
+      <c r="E97">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c0a4e4a486d97a1110d9389a2e7431e168029b9c052c0a4eb43d8fa5c4426a9d</t>
+        </is>
+      </c>
+      <c r="C98">
+        <v>26174</v>
+      </c>
+      <c r="D98">
+        <v>390</v>
+      </c>
+      <c r="E98">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eff88854444211d4122afd5dbd41a0a7a0fe67d6ce77a31d1c8830a9d9763f87</t>
+        </is>
+      </c>
+      <c r="C99">
+        <v>25577</v>
+      </c>
+      <c r="D99">
+        <v>390</v>
+      </c>
+      <c r="E99">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b8d0f7563abf34ebc420f8dafdeb85ed1cfa6f83512cb672c97e3d10b9cb6bf0</t>
+        </is>
+      </c>
+      <c r="C100">
+        <v>71261</v>
+      </c>
+      <c r="D100">
+        <v>1280</v>
+      </c>
+      <c r="E100">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">55ad7a58c0897a189213daaba6caa2025c678759eb1edf9c4da477a6c06f59cd</t>
+        </is>
+      </c>
+      <c r="C101">
+        <v>70274</v>
+      </c>
+      <c r="D101">
+        <v>1280</v>
+      </c>
+      <c r="E101">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d36f2191acc1ba8eb7904ed6cd8ddb3657eab1d1a5b373a17e5318ce79a757c1</t>
+        </is>
+      </c>
+      <c r="C102">
+        <v>35703</v>
+      </c>
+      <c r="D102">
+        <v>390</v>
+      </c>
+      <c r="E102">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fe58d45ede35fd58c1dadaf9ddd7bf7c405e534912bb54153ce6068c92595c6f</t>
+        </is>
+      </c>
+      <c r="C103">
+        <v>34868</v>
+      </c>
+      <c r="D103">
+        <v>390</v>
+      </c>
+      <c r="E103">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34e628e3ffaa2f7f0d7de149e187185c15818fe9ae67b96c928093f186de5fef</t>
+        </is>
+      </c>
+      <c r="C104">
+        <v>35402</v>
+      </c>
+      <c r="D104">
+        <v>390</v>
+      </c>
+      <c r="E104">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bef7ce282a47256d80c1d2b28cdd2ef3d6111ad032d2d11e4bab46539525aec</t>
+        </is>
+      </c>
+      <c r="C105">
+        <v>34434</v>
+      </c>
+      <c r="D105">
+        <v>390</v>
+      </c>
+      <c r="E105">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d3fd6d485d450857ca65082ef91633989044439ab1ef6670652aa5679af1be24</t>
+        </is>
+      </c>
+      <c r="C106">
+        <v>79652</v>
+      </c>
+      <c r="D106">
+        <v>1280</v>
+      </c>
+      <c r="E106">
+        <v>900</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H106">
+        <v>15</v>
+      </c>
+      <c r="I106">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f9eacb23b698618807b651be715db2676b6a8521c561729868f7e0c2260cd1e3</t>
+        </is>
+      </c>
+      <c r="C107">
+        <v>79027</v>
+      </c>
+      <c r="D107">
+        <v>1280</v>
+      </c>
+      <c r="E107">
+        <v>900</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H107">
+        <v>12</v>
+      </c>
+      <c r="I107">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">59953ec07884149c848c5f7f1dc7e6c3f451e5f2bcdd742c2300df96bb1d0f23</t>
+        </is>
+      </c>
+      <c r="C108">
+        <v>41766</v>
+      </c>
+      <c r="D108">
+        <v>390</v>
+      </c>
+      <c r="E108">
+        <v>844</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H108">
+        <v>15</v>
+      </c>
+      <c r="I108">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dbff11dec9d4c901f619d95f2a93bc0928d69ab322286369cd939ddac947d18c</t>
+        </is>
+      </c>
+      <c r="C109">
+        <v>41291</v>
+      </c>
+      <c r="D109">
+        <v>390</v>
+      </c>
+      <c r="E109">
+        <v>844</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-06-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H109">
+        <v>12</v>
+      </c>
+      <c r="I109">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7ddd736539fee331b093308c0dd1ff4c85e8476fc5a9be29c3b24476bb791f4c</t>
+        </is>
+      </c>
+      <c r="C110">
+        <v>70014</v>
+      </c>
+      <c r="D110">
+        <v>1280</v>
+      </c>
+      <c r="E110">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9e8b869d90fb1dbb3d61bc5165794e4c0d50d7003d3607378e091755b050f704</t>
+        </is>
+      </c>
+      <c r="C111">
+        <v>69039</v>
+      </c>
+      <c r="D111">
+        <v>1280</v>
+      </c>
+      <c r="E111">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72b2894e5a5204a913f362c7be193442de97ece5db425a294540f17c18cf7520</t>
+        </is>
+      </c>
+      <c r="C112">
+        <v>41587</v>
+      </c>
+      <c r="D112">
+        <v>390</v>
+      </c>
+      <c r="E112">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a48727c6f46ce1f3c40512a14cfaab32aa9233280c3d8ace4c42901f8fc54eab</t>
+        </is>
+      </c>
+      <c r="C113">
+        <v>41014</v>
+      </c>
+      <c r="D113">
+        <v>390</v>
+      </c>
+      <c r="E113">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b7864d59b1827f608dd181fd4a7a8f2ef7885da0186f6989df71d8889561a104</t>
+        </is>
+      </c>
+      <c r="C114">
+        <v>79828</v>
+      </c>
+      <c r="D114">
+        <v>1280</v>
+      </c>
+      <c r="E114">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">375df600642661f45f6c45ac87130cbff239f2bf42e51ac0ee5266150fc45a1e</t>
+        </is>
+      </c>
+      <c r="C115">
+        <v>79048</v>
+      </c>
+      <c r="D115">
+        <v>1280</v>
+      </c>
+      <c r="E115">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cd02bc6f7f5df890678b955bfd4e61edaf7505eb35ab970ea2fe36349adc5047</t>
+        </is>
+      </c>
+      <c r="C116">
+        <v>41809</v>
+      </c>
+      <c r="D116">
+        <v>390</v>
+      </c>
+      <c r="E116">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ecebdc699bdf88b23686cc1a1591bcf4a0785aacd44aea5a6329b73d4605c24f</t>
+        </is>
+      </c>
+      <c r="C117">
+        <v>41085</v>
+      </c>
+      <c r="D117">
+        <v>390</v>
+      </c>
+      <c r="E117">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">523fd79e8946c26bc4a59fac57a92eb8d28ce66d21639703ee326fda4e9d9190</t>
+        </is>
+      </c>
+      <c r="C118">
+        <v>31841</v>
+      </c>
+      <c r="D118">
+        <v>1280</v>
+      </c>
+      <c r="E118">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8837f9997b6800ec556339037a6b17f9a3345b59b0e0ee89f6b3891e840b1d93</t>
+        </is>
+      </c>
+      <c r="C119">
+        <v>31656</v>
+      </c>
+      <c r="D119">
+        <v>1280</v>
+      </c>
+      <c r="E119">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c0a4e4a486d97a1110d9389a2e7431e168029b9c052c0a4eb43d8fa5c4426a9d</t>
+        </is>
+      </c>
+      <c r="C120">
+        <v>26174</v>
+      </c>
+      <c r="D120">
+        <v>390</v>
+      </c>
+      <c r="E120">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eff88854444211d4122afd5dbd41a0a7a0fe67d6ce77a31d1c8830a9d9763f87</t>
+        </is>
+      </c>
+      <c r="C121">
+        <v>25577</v>
+      </c>
+      <c r="D121">
+        <v>390</v>
+      </c>
+      <c r="E121">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d6d5b12d707c052079a62c65d7b56d4b5ae5d4884a3517b3c177761e5105aaed</t>
+        </is>
+      </c>
+      <c r="C122">
+        <v>71436</v>
+      </c>
+      <c r="D122">
+        <v>1280</v>
+      </c>
+      <c r="E122">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e6c8872e35479263711d5987100ae7653be0182a0aa3c6f8c3bb07c9d3b6290f</t>
+        </is>
+      </c>
+      <c r="C123">
+        <v>70292</v>
+      </c>
+      <c r="D123">
+        <v>1280</v>
+      </c>
+      <c r="E123">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e733d102a61356b24fb3dcbc448b41f0a8b5e57b0cae0a10a86efc8798ba5d03</t>
+        </is>
+      </c>
+      <c r="C124">
+        <v>35746</v>
+      </c>
+      <c r="D124">
+        <v>390</v>
+      </c>
+      <c r="E124">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7379fb43401414f4dcac11dbeb2aadf257845c7ea387a466d1e9cd2878111851</t>
+        </is>
+      </c>
+      <c r="C125">
+        <v>34667</v>
+      </c>
+      <c r="D125">
+        <v>390</v>
+      </c>
+      <c r="E125">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34e628e3ffaa2f7f0d7de149e187185c15818fe9ae67b96c928093f186de5fef</t>
+        </is>
+      </c>
+      <c r="C126">
+        <v>35402</v>
+      </c>
+      <c r="D126">
+        <v>390</v>
+      </c>
+      <c r="E126">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bef7ce282a47256d80c1d2b28cdd2ef3d6111ad032d2d11e4bab46539525aec</t>
+        </is>
+      </c>
+      <c r="C127">
+        <v>34434</v>
+      </c>
+      <c r="D127">
+        <v>390</v>
+      </c>
+      <c r="E127">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6e3555dfe49824da23ce3c89243d88c128877856daa52aeb4a0a5bd0f36d61d0</t>
+        </is>
+      </c>
+      <c r="C128">
+        <v>79828</v>
+      </c>
+      <c r="D128">
+        <v>1280</v>
+      </c>
+      <c r="E128">
+        <v>900</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H128">
+        <v>15</v>
+      </c>
+      <c r="I128">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ff73028f91f720a172870c2cb1afade85828f9231b05b800843d9b644a05c02c</t>
+        </is>
+      </c>
+      <c r="C129">
+        <v>79043</v>
+      </c>
+      <c r="D129">
+        <v>1280</v>
+      </c>
+      <c r="E129">
+        <v>900</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H129">
+        <v>12</v>
+      </c>
+      <c r="I129">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d7584edfccb02fc7650b31e2b77ace0a76b09ce56f3d9b01033d62f00ee4e26f</t>
+        </is>
+      </c>
+      <c r="C130">
+        <v>41809</v>
+      </c>
+      <c r="D130">
+        <v>390</v>
+      </c>
+      <c r="E130">
+        <v>844</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H130">
+        <v>15</v>
+      </c>
+      <c r="I130">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6ffabcfb695a0e4cc17cf4302dda11be547f99d7f7cea3549b44385dba99b0cc</t>
+        </is>
+      </c>
+      <c r="C131">
+        <v>41077</v>
+      </c>
+      <c r="D131">
+        <v>390</v>
+      </c>
+      <c r="E131">
+        <v>844</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near</t>
+        </is>
+      </c>
+      <c r="H131">
+        <v>12</v>
+      </c>
+      <c r="I131">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I65"/>
+  <autoFilter ref="A1:I131"/>
 </worksheet>
 </file>
 
@@ -8776,7 +10420,7 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="4" max="4" width="59" customWidth="1"/>
     <col min="5" max="5" width="59" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="61" customWidth="1"/>
@@ -8837,12 +10481,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -8874,12 +10518,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -8911,12 +10555,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -8948,12 +10592,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -8985,12 +10629,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -9022,12 +10666,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -9059,12 +10703,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -9096,12 +10740,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -9133,12 +10777,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -9170,12 +10814,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -9207,12 +10851,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -9244,12 +10888,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-02-before-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -9271,7 +10915,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="1" max="1" width="45" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
@@ -9306,7 +10950,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">599 tests / 47 files; source-string recovery guard updated for same held/live/no-code condition and native disclosure</t>
+          <t xml:space="preserve">599tests/47files on final single-pane implementation, including explicit-selection wrapper; /tmp/kynotes-single-nav-unit-final.log</t>
         </is>
       </c>
     </row>
@@ -9340,14 +10984,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/12 on a fresh default e2e server; capture outputs isolated from suite traces</t>
+          <t xml:space="preserve">12/12 full fresh-server browser tests on final implementation; /tmp/kynotes-single-nav-browser-verified.log. Covers saved content, team keys, startup race, notebook management, keyboard disclosure and phone reachability.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage04 capture and regressions</t>
+          <t xml:space="preserve">Stage07 single-pane capture and regressions</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9357,7 +11001,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 captures; first picker row in viewport, same/different-id focus, held PUT dirty state and reload persistence, recovery warning/action keyboard disclosure</t>
+          <t xml:space="preserve">22captures/18unique, including4empty and2desktop management views. Single240px pane geometry, phone chooser, same/different pagefocus, heldPUTsave and recoverykeyboard pass; /tmp/kynotes-single-nav-capture-verified.log.</t>
         </is>
       </c>
     </row>
@@ -9408,7 +11052,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two clean private extractions of staged source tree cd1200e4379252f86bebd63e48f41ad324a4d016; CGO_ENABLED=0 go build -trimpath, release0.0.0; both binary SHA256 71b0e7716ce571a6b3284b0ad6b6c935f2809fd141d82d17cd969f80d260eb21. No product/build input changed afterward.</t>
+          <t xml:space="preserve">Verified final-source treee9cd105a6896cd4fc35828ebae05e0612836353d; two clean private extractions, CGO_ENABLED=0 -trimpath release0.0.0; both binarySHA256 d15e35eceb80b338347561f3aad24f03578e71525e16cf832bdac4978afd8558. Product inputs unchanged afterward.</t>
         </is>
       </c>
     </row>
@@ -9510,7 +11154,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Final image build,14-step probe and apply-setup pass; logs /tmp/kynotes-eight-{docker,probe,container-setup}-final.log</t>
+          <t xml:space="preserve">Final verified-source image build,14-step probe and setup passed; /tmp/kynotes-single-nav-{docker,probe,setup}-verified.log</t>
         </is>
       </c>
     </row>
@@ -9578,7 +11222,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Real18101 fixture: owner login, open Launch checklist,390x844 page chooser; all4rows visible y355–636, editor hidden while choosing, zero horizontal overflow; computed body15px/22.5px Space strong ink. Native snapshots/geometry can update asynchronously; scored PNGs remain the recorded Chromium156 set.</t>
+          <t xml:space="preserve">Final18104 fixture, signed-in owner. Native1280px: page listx0/editorx240 with management hidden; opening management gives sidebarx0/width240, hides page list and retains editorx240; zero horizontal overflow. Browser automation separately covers390x844 and keyboard/focus/save paths.</t>
         </is>
       </c>
     </row>
@@ -9684,7 +11328,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage04 after; all earlier inputs retained</t>
+          <t xml:space="preserve">Stage07 after; all earlier inputs retained</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: link the single-navigation follow-up pull request
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -11448,8 +11448,30 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Busnes-app/KyNotes-server</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://github.com/Busnes-app/KyNotes-server/pull/119</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ui/notes-eight</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-up after merged118: single left navigation pane, owner6 record and fresh round4 evidence; no merge/deployment</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D4"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
expose first notebook creation in the empty workspace
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -235,12 +235,57 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Pending</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deferred</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
+  <autoFilter ref="A1:I6"/>
 </worksheet>
 </file>
 
@@ -9409,7 +9454,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="59" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
   </cols>
@@ -12735,8 +12780,630 @@
         <v>4</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7ddd736539fee331b093308c0dd1ff4c85e8476fc5a9be29c3b24476bb791f4c</t>
+        </is>
+      </c>
+      <c r="C132">
+        <v>70014</v>
+      </c>
+      <c r="D132">
+        <v>1280</v>
+      </c>
+      <c r="E132">
+        <v>900</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H132">
+        <v>0</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9e8b869d90fb1dbb3d61bc5165794e4c0d50d7003d3607378e091755b050f704</t>
+        </is>
+      </c>
+      <c r="C133">
+        <v>69039</v>
+      </c>
+      <c r="D133">
+        <v>1280</v>
+      </c>
+      <c r="E133">
+        <v>900</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H133">
+        <v>0</v>
+      </c>
+      <c r="I133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">72b2894e5a5204a913f362c7be193442de97ece5db425a294540f17c18cf7520</t>
+        </is>
+      </c>
+      <c r="C134">
+        <v>41587</v>
+      </c>
+      <c r="D134">
+        <v>390</v>
+      </c>
+      <c r="E134">
+        <v>844</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H134">
+        <v>0</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a48727c6f46ce1f3c40512a14cfaab32aa9233280c3d8ace4c42901f8fc54eab</t>
+        </is>
+      </c>
+      <c r="C135">
+        <v>41014</v>
+      </c>
+      <c r="D135">
+        <v>390</v>
+      </c>
+      <c r="E135">
+        <v>844</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H135">
+        <v>0</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05a9187350416aa3b1cf40880e5ff5646635ab0069ff1d9e87a7166e58a9256d</t>
+        </is>
+      </c>
+      <c r="C136">
+        <v>79937</v>
+      </c>
+      <c r="D136">
+        <v>1280</v>
+      </c>
+      <c r="E136">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c36eec5234ec3d74e1e16082fc58cd1308469f106f00a5ca3aca907543b96950</t>
+        </is>
+      </c>
+      <c r="C137">
+        <v>78979</v>
+      </c>
+      <c r="D137">
+        <v>1280</v>
+      </c>
+      <c r="E137">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bb72aadfd10dc888385c654c25d2a8b8ea47921b0ad8c59fe46a392dcb4e1ab4</t>
+        </is>
+      </c>
+      <c r="C138">
+        <v>42089</v>
+      </c>
+      <c r="D138">
+        <v>390</v>
+      </c>
+      <c r="E138">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1a2066d9b8c44ddd297e2e0485929fa4cb69826f3625a1049dd8082a6d1dd5b5</t>
+        </is>
+      </c>
+      <c r="C139">
+        <v>41294</v>
+      </c>
+      <c r="D139">
+        <v>390</v>
+      </c>
+      <c r="E139">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">67688db5fc72189cbcb4af5f0b559d69f96f9bfb385688d421e3cc3456c5c4cb</t>
+        </is>
+      </c>
+      <c r="C140">
+        <v>35401</v>
+      </c>
+      <c r="D140">
+        <v>1280</v>
+      </c>
+      <c r="E140">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ad6a6b843ad7f0327b7ccdf93ffdcde7eb4cce8137e1b33bad03a7b3dd3b92c9</t>
+        </is>
+      </c>
+      <c r="C141">
+        <v>35203</v>
+      </c>
+      <c r="D141">
+        <v>1280</v>
+      </c>
+      <c r="E141">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf5201ca043db6727c20daf1d4f15e4009bf3193d0405c5088afc94dcc7be040</t>
+        </is>
+      </c>
+      <c r="C142">
+        <v>29255</v>
+      </c>
+      <c r="D142">
+        <v>390</v>
+      </c>
+      <c r="E142">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38ea2008811c859c52500f203c7be160abca2f187368625cda147a4f72257320</t>
+        </is>
+      </c>
+      <c r="C143">
+        <v>28609</v>
+      </c>
+      <c r="D143">
+        <v>390</v>
+      </c>
+      <c r="E143">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ff86ee660c83becc1d81e5998d5c4c6b42d26c8621d7d7f0fcde69fa070151b3</t>
+        </is>
+      </c>
+      <c r="C144">
+        <v>71547</v>
+      </c>
+      <c r="D144">
+        <v>1280</v>
+      </c>
+      <c r="E144">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8085c2811af8b5ef488674e105f72ebed314b82f007095ad2ea1949dd6780d0c</t>
+        </is>
+      </c>
+      <c r="C145">
+        <v>70227</v>
+      </c>
+      <c r="D145">
+        <v>1280</v>
+      </c>
+      <c r="E145">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">953ce6476d79b4c6b0b2b0dfc49d2e9dc2d4ef841dbfbac1d5b053d262e98158</t>
+        </is>
+      </c>
+      <c r="C146">
+        <v>36029</v>
+      </c>
+      <c r="D146">
+        <v>390</v>
+      </c>
+      <c r="E146">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27238c23a549a97252fe2140492add53efe15a7d3f2e4f1f788def3f95dbe36c</t>
+        </is>
+      </c>
+      <c r="C147">
+        <v>34864</v>
+      </c>
+      <c r="D147">
+        <v>390</v>
+      </c>
+      <c r="E147">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34e628e3ffaa2f7f0d7de149e187185c15818fe9ae67b96c928093f186de5fef</t>
+        </is>
+      </c>
+      <c r="C148">
+        <v>35402</v>
+      </c>
+      <c r="D148">
+        <v>390</v>
+      </c>
+      <c r="E148">
+        <v>844</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H148">
+        <v>0</v>
+      </c>
+      <c r="I148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bef7ce282a47256d80c1d2b28cdd2ef3d6111ad032d2d11e4bab46539525aec</t>
+        </is>
+      </c>
+      <c r="C149">
+        <v>34434</v>
+      </c>
+      <c r="D149">
+        <v>390</v>
+      </c>
+      <c r="E149">
+        <v>844</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-05-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H149">
+        <v>0</v>
+      </c>
+      <c r="I149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9a046b247b82cceb17ff22261a8ba1dc0c8d25ea0d2028ac2beac46819400340</t>
+        </is>
+      </c>
+      <c r="C150">
+        <v>79938</v>
+      </c>
+      <c r="D150">
+        <v>1280</v>
+      </c>
+      <c r="E150">
+        <v>900</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (caret rasterization)</t>
+        </is>
+      </c>
+      <c r="H150">
+        <v>15</v>
+      </c>
+      <c r="I150">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7745dbaf57c287698bd7cfd00e27989fa20e994c1b94b359cc31c702fff9e538</t>
+        </is>
+      </c>
+      <c r="C151">
+        <v>78973</v>
+      </c>
+      <c r="D151">
+        <v>1280</v>
+      </c>
+      <c r="E151">
+        <v>900</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (caret rasterization)</t>
+        </is>
+      </c>
+      <c r="H151">
+        <v>12</v>
+      </c>
+      <c r="I151">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cc49a9988c98e5aed7af5d30879364a85d0f1472c1f0bb3032a19b9a449935f8</t>
+        </is>
+      </c>
+      <c r="C152">
+        <v>42089</v>
+      </c>
+      <c r="D152">
+        <v>390</v>
+      </c>
+      <c r="E152">
+        <v>844</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (caret rasterization)</t>
+        </is>
+      </c>
+      <c r="H152">
+        <v>15</v>
+      </c>
+      <c r="I152">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4d062804312511d8e11664d44ec3c95f932da960bc226f7254f3669e19850e3e</t>
+        </is>
+      </c>
+      <c r="C153">
+        <v>41285</v>
+      </c>
+      <c r="D153">
+        <v>390</v>
+      </c>
+      <c r="E153">
+        <v>844</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (caret rasterization)</t>
+        </is>
+      </c>
+      <c r="H153">
+        <v>12</v>
+      </c>
+      <c r="I153">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I131"/>
+  <autoFilter ref="A1:I153"/>
 </worksheet>
 </file>
 
@@ -12807,12 +13474,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -12829,7 +13496,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">appearance</t>
+          <t xml:space="preserve">empty</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12844,12 +13511,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -12866,7 +13533,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">editor</t>
+          <t xml:space="preserve">appearance</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12876,17 +13543,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">dark</t>
+          <t xml:space="preserve">light</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -12903,7 +13570,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">appearance</t>
+          <t xml:space="preserve">navigation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -12913,27 +13580,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">dark</t>
+          <t xml:space="preserve">light</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">True</t>
+          <t xml:space="preserve">False</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fresh accounts change initials/times; same content</t>
+          <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
         </is>
       </c>
     </row>
@@ -12945,22 +13612,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">mobile</t>
+          <t xml:space="preserve">desktop</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">light</t>
+          <t xml:space="preserve">dark</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -12977,27 +13644,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">appearance</t>
+          <t xml:space="preserve">empty</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">mobile</t>
+          <t xml:space="preserve">desktop</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">light</t>
+          <t xml:space="preserve">dark</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -13014,37 +13681,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pages</t>
+          <t xml:space="preserve">appearance</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mobile</t>
+          <t xml:space="preserve">desktop</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">light</t>
+          <t xml:space="preserve">dark</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">False</t>
+          <t xml:space="preserve">True</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
+          <t xml:space="preserve">Fresh accounts change initials/times; same content</t>
         </is>
       </c>
     </row>
@@ -13056,22 +13723,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">mobile</t>
+          <t xml:space="preserve">desktop</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">light</t>
+          <t xml:space="preserve">dark</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -13098,17 +13765,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">dark</t>
+          <t xml:space="preserve">light</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -13125,7 +13792,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">appearance</t>
+          <t xml:space="preserve">empty</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -13135,17 +13802,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">dark</t>
+          <t xml:space="preserve">light</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -13162,7 +13829,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">pages</t>
+          <t xml:space="preserve">appearance</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -13172,77 +13839,299 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">dark</t>
+          <t xml:space="preserve">light</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">False</t>
+          <t xml:space="preserve">True</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
+          <t xml:space="preserve">Fresh accounts change initials/times; same content</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t xml:space="preserve">pages</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mobile</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">light</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t xml:space="preserve">navigation</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t xml:space="preserve">mobile</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">light</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">editor</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mobile</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t xml:space="preserve">dark</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">screenshots/kynotes-04-after-navigation-mobile-dark.png</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fresh accounts change initials/times; same content</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">empty</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mobile</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dark</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fresh accounts change initials/times; same content</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">appearance</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mobile</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dark</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fresh accounts change initials/times; same content</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pages</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mobile</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dark</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-07-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">navigation</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mobile</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dark</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t xml:space="preserve">screenshots/kynotes-07-after-navigation-mobile-dark.png</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-08-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t xml:space="preserve">False</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t xml:space="preserve">Different navigation state; no controlled improvement claim</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:G19"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="37" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
+    <col min="2" max="2" width="58" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
@@ -13276,7 +14165,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">599tests/47files on final single-pane implementation, including explicit-selection wrapper; /tmp/kynotes-single-nav-unit-final.log</t>
+          <t xml:space="preserve">599 tests/47 files; /tmp/kynotes-first-notebook-unit.log.</t>
         </is>
       </c>
     </row>
@@ -13293,7 +14182,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">npm run build --prefix web; exact regenerated embed; existing 603kB lazy BlockNote chunk size warning retained</t>
+          <t xml:space="preserve">npm run build --prefix web; rsync generated assets with deletion; diff -qr web/dist internal/web/dist clean. Existing 603kB lazy BlockNote warning.</t>
         </is>
       </c>
     </row>
@@ -13310,7 +14199,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/12 full fresh-server browser tests on final implementation; /tmp/kynotes-single-nav-browser-verified.log. Covers saved content, team keys, startup race, notebook management, keyboard disclosure and phone reachability.</t>
+          <t xml:space="preserve">12/12 full fresh-server tests; /tmp/kynotes-first-notebook-browser.log. Final stage08 separately runs exact current capture driver with explicit creation-focus wait.</t>
         </is>
       </c>
     </row>
@@ -13344,7 +14233,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">go build ./...; go vet ./...; gofmt clean; go test ./internal/web; diff -qr web/dist internal/web/dist</t>
+          <t xml:space="preserve">go build; go vet ./...; go test ./internal/web; diff -qr web/dist internal/web/dist clean; no Go source changes.</t>
         </is>
       </c>
     </row>
@@ -13378,7 +14267,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verified final-source treee9cd105a6896cd4fc35828ebae05e0612836353d; two clean private extractions, CGO_ENABLED=0 -trimpath release0.0.0; both binarySHA256 d15e35eceb80b338347561f3aad24f03578e71525e16cf832bdac4978afd8558. Product inputs unchanged afterward.</t>
+          <t xml:space="preserve">Current stage08 product source in staged tree a5d5b228a05673c06ee59349b7ff50b259a713a8; two private clean git-archive builds, CGO_ENABLED=0 -trimpath release0.0.0. Identical SHA256 f899bddbf75e2dc615262ad1ee085b6657c6d14f7075989ebb77679e964a8be9. /tmp/kynotes-first-notebook-repeatability.log; later evidence-only metadata cannot affect binary.</t>
         </is>
       </c>
     </row>
@@ -13480,7 +14369,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Final verified-source image build,14-step probe and setup passed; /tmp/kynotes-single-nav-{docker,probe,setup}-verified.log</t>
+          <t xml:space="preserve">Current-source kynotes-first-notebook:r5 built;14-step probe and apply-setup pass. /tmp/kynotes-first-notebook-{docker,probe,setup}.log. Initial probe invocation used unsupported docker:&lt;name&gt;; corrected to documented docker transport and fixed container name.</t>
         </is>
       </c>
     </row>
@@ -13492,12 +14381,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 documented exceptions</t>
+          <t xml:space="preserve">pass on changed target; existing CSS exceptions retained</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Semantic conflict/key-warning rail (3px) and user-colored section top border (legacy4px rule overridden to2px). No blanket suppression; raw detector.json retained</t>
+          <t xml:space="preserve">Current main.tsx detector returned []; /tmp/kynotes-first-notebook-detector.json. Existing CSS exceptions remain documented in detector.json.</t>
         </is>
       </c>
     </row>
@@ -13548,7 +14437,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Final18104 fixture, signed-in owner. Native1280px: page listx0/editorx240 with management hidden; opening management gives sidebarx0/width240, hides page list and retains editorx240; zero horizontal overflow. Browser automation separately covers390x844 and keyboard/focus/save paths.</t>
+          <t xml:space="preserve">Current served bundle on18105: desktop management x0,width240; pages hidden; editor x240; zero overflow. Work queue closes management and activeElement is Notebooks and account. Stage08 Chromium156 separately tests first-notebook creation and390px reachability. Native input tool required DOM input events for login; no source/security change.</t>
         </is>
       </c>
     </row>
@@ -13586,8 +14475,25 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage08 first-notebook capture and regressions</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pass</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22 captures/18 unique on fresh18106 fixture; /tmp/kynotes-first-notebook-capture-final.log. New notebook above phone fold in both themes, real creation, key/recovery guidance, one-pane geometry, immediate selection focus, held-save/reload and Work queue focus. Initial capture failed on a test focus race; explicit wait for completed navigation corrected it before any round5 delegation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C20"/>
+  <autoFilter ref="A1:C21"/>
 </worksheet>
 </file>
 
@@ -13654,7 +14560,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage07 after; all earlier inputs retained</t>
+          <t xml:space="preserve">Stage08 after; all earlier inputs retained</t>
         </is>
       </c>
     </row>
@@ -13792,7 +14698,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Follow-up after merged118: single left navigation pane, owner6 record and fresh round4 evidence; no merge/deployment</t>
+          <t xml:space="preserve">Follow-up after merged118: one left navigation pane, visible first-notebook action, owner6 record and fresh council evidence; no merge/deployment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh first-notebook review provenance and delivery
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -14654,7 +14654,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shared0.4.2 status and field contrast; staged consumer adoption</t>
+          <t xml:space="preserve">Merged shared0.4.2 status and field contrast; staged consumer adoption</t>
         </is>
       </c>
     </row>
@@ -14676,7 +14676,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Editor, phone navigation and frozen council evidence; no merge/deployment</t>
+          <t xml:space="preserve">Merged original editor/phone-navigation pass and frozen council evidence; merged externally, not by this agent</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
theme placeholders and clarify workspace actions
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -358,12 +358,57 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Pending</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deferred</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I9"/>
 </worksheet>
 </file>
 
@@ -22464,8 +22509,662 @@
         <v>4</v>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c75e0f370c7b318a30b96856e857ddee878c559633886009ce2f34bb8916cc89</t>
+        </is>
+      </c>
+      <c r="C198">
+        <v>69755</v>
+      </c>
+      <c r="D198">
+        <v>1280</v>
+      </c>
+      <c r="E198">
+        <v>900</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H198">
+        <v>0</v>
+      </c>
+      <c r="I198">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e65157f29c09998407a3643285cd11506950fc1784b9e24c48f27a5bc98e1fe</t>
+        </is>
+      </c>
+      <c r="C199">
+        <v>68773</v>
+      </c>
+      <c r="D199">
+        <v>1280</v>
+      </c>
+      <c r="E199">
+        <v>900</v>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H199">
+        <v>0</v>
+      </c>
+      <c r="I199">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d56fb7f8861c404dd66b7540a14a792b09ebd35b4dd87f1cc50e65a0f048d4c2</t>
+        </is>
+      </c>
+      <c r="C200">
+        <v>41329</v>
+      </c>
+      <c r="D200">
+        <v>390</v>
+      </c>
+      <c r="E200">
+        <v>844</v>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H200">
+        <v>0</v>
+      </c>
+      <c r="I200">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">273573674ce231a8ef3ed13abe078611803aa2db45a6db081ba01488b7400bc1</t>
+        </is>
+      </c>
+      <c r="C201">
+        <v>40731</v>
+      </c>
+      <c r="D201">
+        <v>390</v>
+      </c>
+      <c r="E201">
+        <v>844</v>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H201">
+        <v>0</v>
+      </c>
+      <c r="I201">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0f33d1256160273e4b458a64a8bc566e59fabd59d7d80df8ed79a3910c0e3348</t>
+        </is>
+      </c>
+      <c r="C202">
+        <v>78087</v>
+      </c>
+      <c r="D202">
+        <v>1280</v>
+      </c>
+      <c r="E202">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4f0c64b0d7aae9145b0186fb669be5e239bec004dc1dacc70f2375487698be36</t>
+        </is>
+      </c>
+      <c r="C203">
+        <v>77256</v>
+      </c>
+      <c r="D203">
+        <v>1280</v>
+      </c>
+      <c r="E203">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5f5427237b0fee184c2f04c684477e49474258868ea5c6de44b125ae07870d7e</t>
+        </is>
+      </c>
+      <c r="C204">
+        <v>41293</v>
+      </c>
+      <c r="D204">
+        <v>390</v>
+      </c>
+      <c r="E204">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a0f529227d1bf15d3bcbc107b34205569a0a15c3ee7fbf662f5bb0f7c2cadee6</t>
+        </is>
+      </c>
+      <c r="C205">
+        <v>40518</v>
+      </c>
+      <c r="D205">
+        <v>390</v>
+      </c>
+      <c r="E205">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bb7c1e9f1bb2e595fef91ad00eb7b483b20fdf7832825094759ef38fc277b1a</t>
+        </is>
+      </c>
+      <c r="C206">
+        <v>32909</v>
+      </c>
+      <c r="D206">
+        <v>1280</v>
+      </c>
+      <c r="E206">
+        <v>900</v>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H206">
+        <v>0</v>
+      </c>
+      <c r="I206">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70340422c86d96f05b2de950ae87c2a10ea4d744d0e9a428914a56c6b7b3a3c5</t>
+        </is>
+      </c>
+      <c r="C207">
+        <v>32544</v>
+      </c>
+      <c r="D207">
+        <v>1280</v>
+      </c>
+      <c r="E207">
+        <v>900</v>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H207">
+        <v>0</v>
+      </c>
+      <c r="I207">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">854dff5ab7a8e69b5ae28642c0d16a04b360c94deb43f848eda89a6dd3907058</t>
+        </is>
+      </c>
+      <c r="C208">
+        <v>25542</v>
+      </c>
+      <c r="D208">
+        <v>390</v>
+      </c>
+      <c r="E208">
+        <v>844</v>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H208">
+        <v>0</v>
+      </c>
+      <c r="I208">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">97ec527b9dc09c37850e51690609855720f60a32c02d0281a0f54b4173eb999f</t>
+        </is>
+      </c>
+      <c r="C209">
+        <v>25146</v>
+      </c>
+      <c r="D209">
+        <v>390</v>
+      </c>
+      <c r="E209">
+        <v>844</v>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H209">
+        <v>0</v>
+      </c>
+      <c r="I209">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d76819360e250995d78782fbdfc1328c7e5e1f1fb271d29e578b3e1dede821c4</t>
+        </is>
+      </c>
+      <c r="C210">
+        <v>69978</v>
+      </c>
+      <c r="D210">
+        <v>1280</v>
+      </c>
+      <c r="E210">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18c8d8b197c34dcd40ce8acf26c7a7d9a582d5b7818a8a54a10b71bc823e510b</t>
+        </is>
+      </c>
+      <c r="C211">
+        <v>69098</v>
+      </c>
+      <c r="D211">
+        <v>1280</v>
+      </c>
+      <c r="E211">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2695ba90d7a666dfcd197d4d0227c58f606bf5957b536937b8051fc15b235b7a</t>
+        </is>
+      </c>
+      <c r="C212">
+        <v>35435</v>
+      </c>
+      <c r="D212">
+        <v>390</v>
+      </c>
+      <c r="E212">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d1c5027ccc51ed7fef1f882a402d4a7d9663057fcb1d69f721730c2b5c9c3210</t>
+        </is>
+      </c>
+      <c r="C213">
+        <v>34596</v>
+      </c>
+      <c r="D213">
+        <v>390</v>
+      </c>
+      <c r="E213">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bb5e059ba4f728b61a9cff2b4fdbfc826bc4d4c72035e900d888e599acf9bf8f</t>
+        </is>
+      </c>
+      <c r="C214">
+        <v>34827</v>
+      </c>
+      <c r="D214">
+        <v>390</v>
+      </c>
+      <c r="E214">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4dcbdefa1ee0ece84d7c82481c3490d8ba6a57e75d3469b813c3f752e046368b</t>
+        </is>
+      </c>
+      <c r="C215">
+        <v>33894</v>
+      </c>
+      <c r="D215">
+        <v>390</v>
+      </c>
+      <c r="E215">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bd1c06f66a7d3c4b0f4777db669816604c382cbdb30286eb19ef8f8b14897cc5</t>
+        </is>
+      </c>
+      <c r="C216">
+        <v>78088</v>
+      </c>
+      <c r="D216">
+        <v>1280</v>
+      </c>
+      <c r="E216">
+        <v>900</v>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H216">
+        <v>15</v>
+      </c>
+      <c r="I216">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">86afbd938d4db9444e78b3e447385d218a158ca2d3ad7dbea0343b448ab11db7</t>
+        </is>
+      </c>
+      <c r="C217">
+        <v>77248</v>
+      </c>
+      <c r="D217">
+        <v>1280</v>
+      </c>
+      <c r="E217">
+        <v>900</v>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H217">
+        <v>12</v>
+      </c>
+      <c r="I217">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">61a6de77d880cad16d6ba382d6ab3c612985fe6c0c541c8a17e1f655675198ae</t>
+        </is>
+      </c>
+      <c r="C218">
+        <v>41296</v>
+      </c>
+      <c r="D218">
+        <v>390</v>
+      </c>
+      <c r="E218">
+        <v>844</v>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H218">
+        <v>15</v>
+      </c>
+      <c r="I218">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">906d03b0c06762c830261d6cb40e4b4c98509985ba1f73e143de48ace68fbed1</t>
+        </is>
+      </c>
+      <c r="C219">
+        <v>40510</v>
+      </c>
+      <c r="D219">
+        <v>390</v>
+      </c>
+      <c r="E219">
+        <v>844</v>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H219">
+        <v>12</v>
+      </c>
+      <c r="I219">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I197"/>
+  <autoFilter ref="A1:I219"/>
 </worksheet>
 </file>
 
@@ -22536,12 +23235,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -22573,12 +23272,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-empty-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -22610,12 +23309,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -22647,12 +23346,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-navigation-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -22684,12 +23383,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -22721,12 +23420,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-empty-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -22758,12 +23457,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -22795,12 +23494,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-navigation-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -22832,12 +23531,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -22869,12 +23568,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-empty-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -22906,12 +23605,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -22943,12 +23642,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -22980,12 +23679,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -23017,12 +23716,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -23054,12 +23753,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-empty-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-dark.png</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-dark.png</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -23091,12 +23790,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -23128,12 +23827,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -23165,12 +23864,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-09-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -23227,7 +23926,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">599 tests/47 files on round7; /tmp/kynotes-controls-r7-unit.log.</t>
+          <t xml:space="preserve">599 tests/47files on final round8 source; /tmp/kynotes-affordance-r8-unit-final.log.</t>
         </is>
       </c>
     </row>
@@ -23244,7 +23943,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round7 build/TypeScript/exact embed pass; /tmp/kynotes-controls-r7-build.log. Existing603kB lazy BlockNote warning.</t>
+          <t xml:space="preserve">Final round8 TS/build/exact embed pass; /tmp/kynotes-affordance-r8-build-final.log. Existing603kBBlockNote warning.</t>
         </is>
       </c>
     </row>
@@ -23261,7 +23960,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/12 fresh full browser tests, first attempt on round7; /tmp/kynotes-controls-r7-browser.log. No changed application behavior; stage10 also passes the creation/focus/held-save/recovery regressions.</t>
+          <t xml:space="preserve">12/12 fresh-server browsers first attempt on final round8 source; /tmp/kynotes-affordance-r8-browser.log.</t>
         </is>
       </c>
     </row>
@@ -23329,7 +24028,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round7 staged tree d1c6c9af46a321b6c8ac07378828cd0fad6227c5; two private clean archives,CGO_ENABLED=0,-trimpath,release0.0.0. Both SHA256f608e0de3bc4a6fb56099fa2c060741d1a661a5cc52c218c3aa24ee1fe4c2d6c; /tmp/kynotes-controls-r7-repeatability.log. Later report metadata does not affect binary.</t>
+          <t xml:space="preserve">Round8 staged tree9327c94f64ffac83b5354708726364bd1b4df09b; two private clean archives,CGO_ENABLED=0,-trimpath,release0.0.0. BothSHA2564edf95b5bafa4b324967ff8d9ae1db3079deb9f1f1105c1d147c8510186db176; /tmp/kynotes-affordance-r8-repeatability.log. Later evidence/AGENTS metadata cannot affect binary.</t>
         </is>
       </c>
     </row>
@@ -23431,7 +24130,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round7 current-source kynotes-controls:r7 image,14-step probe,setup pass; /tmp/kynotes-controls-r7-{docker,probe,setup}.log.</t>
+          <t xml:space="preserve">Current kynotes-affordance:r8 image,14step probe/setup pass; /tmp/kynotes-affordance-r8-{docker,probe,setup}.log.</t>
         </is>
       </c>
     </row>
@@ -23448,7 +24147,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round7 CSS detector: only semantic key/conflict rail3px and legacy section top4px overridden2px; controls-round7-detector.json. No suppression.</t>
+          <t xml:space="preserve">Round8 changed-source detector only existing semantic warning rail and overridden section-color border; affordance-round8-detector.json.</t>
         </is>
       </c>
     </row>
@@ -23494,12 +24193,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">pass, narrow measurements</t>
+          <t xml:space="preserve">pass, scoped</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">stage10 live18110 at1280x800: representative Save/Search/comment inputs/Comment have14px text,8px radius,equal edges4.5449:1(light) and5.3234:1(dark),heading/search/toggletextx16,overflow0. theme-checks/round7-native-controls.json and darkPNG. These samples do not certify every theme/control/state.</t>
+          <t xml:space="preserve">Old live dark placeholder117grey confirmed. Current18111 three placeholders6.1926:1 light/7.4845:1 dark,section button40x40,toolbar separator1x24,inbox Workqueue path,overflow0. Native section popover opens with both existing options; no content created. theme-checks/round8-native-placeholders.json and lightPNG.</t>
         </is>
       </c>
     </row>
@@ -23605,8 +24304,25 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage11 placeholder/affordance capture and regressions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pass</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22captures/18unique, first attempt22.5s on fresh18111; /tmp/kynotes-affordance-r8-capture.log. Source pins now include CanvasPage.tsx (9files) for the toolbar separator. Same fixtures,viewport/themes and save/focus/recovery checks.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C24"/>
+  <autoFilter ref="A1:C25"/>
 </worksheet>
 </file>
 
@@ -23673,7 +24389,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage10 after; all earlier inputs retained</t>
+          <t xml:space="preserve">Stage11 after; all earlier inputs retained</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: align note controls and phone editor spacing
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -403,8 +403,53 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deferred</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:I10"/>
 </worksheet>
 </file>
 
@@ -25795,8 +25840,630 @@
         <v>4</v>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c75e0f370c7b318a30b96856e857ddee878c559633886009ce2f34bb8916cc89</t>
+        </is>
+      </c>
+      <c r="C220">
+        <v>69755</v>
+      </c>
+      <c r="D220">
+        <v>1280</v>
+      </c>
+      <c r="E220">
+        <v>900</v>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H220">
+        <v>0</v>
+      </c>
+      <c r="I220">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e65157f29c09998407a3643285cd11506950fc1784b9e24c48f27a5bc98e1fe</t>
+        </is>
+      </c>
+      <c r="C221">
+        <v>68773</v>
+      </c>
+      <c r="D221">
+        <v>1280</v>
+      </c>
+      <c r="E221">
+        <v>900</v>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H221">
+        <v>0</v>
+      </c>
+      <c r="I221">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d56fb7f8861c404dd66b7540a14a792b09ebd35b4dd87f1cc50e65a0f048d4c2</t>
+        </is>
+      </c>
+      <c r="C222">
+        <v>41329</v>
+      </c>
+      <c r="D222">
+        <v>390</v>
+      </c>
+      <c r="E222">
+        <v>844</v>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H222">
+        <v>0</v>
+      </c>
+      <c r="I222">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">273573674ce231a8ef3ed13abe078611803aa2db45a6db081ba01488b7400bc1</t>
+        </is>
+      </c>
+      <c r="C223">
+        <v>40731</v>
+      </c>
+      <c r="D223">
+        <v>390</v>
+      </c>
+      <c r="E223">
+        <v>844</v>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H223">
+        <v>0</v>
+      </c>
+      <c r="I223">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f4dc17dc2149368266a44c90313aa93d28d8d109ae84ba5ecb9bc13e38433bf5</t>
+        </is>
+      </c>
+      <c r="C224">
+        <v>78132</v>
+      </c>
+      <c r="D224">
+        <v>1280</v>
+      </c>
+      <c r="E224">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eaee7de84cd1660ceba857d5ff6428dbe96ebe661c0618703ea826f071ee57ed</t>
+        </is>
+      </c>
+      <c r="C225">
+        <v>77284</v>
+      </c>
+      <c r="D225">
+        <v>1280</v>
+      </c>
+      <c r="E225">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e33dd62356cf53287e3655ccc3498c58682d8daa1f00fdf1655299daebd1617</t>
+        </is>
+      </c>
+      <c r="C226">
+        <v>43078</v>
+      </c>
+      <c r="D226">
+        <v>390</v>
+      </c>
+      <c r="E226">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06aa3fceec6e800e52837a619c97345dc771d89b5b7152819a2e4f64251c48f4</t>
+        </is>
+      </c>
+      <c r="C227">
+        <v>42211</v>
+      </c>
+      <c r="D227">
+        <v>390</v>
+      </c>
+      <c r="E227">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bb7c1e9f1bb2e595fef91ad00eb7b483b20fdf7832825094759ef38fc277b1a</t>
+        </is>
+      </c>
+      <c r="C228">
+        <v>32909</v>
+      </c>
+      <c r="D228">
+        <v>1280</v>
+      </c>
+      <c r="E228">
+        <v>900</v>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H228">
+        <v>0</v>
+      </c>
+      <c r="I228">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70340422c86d96f05b2de950ae87c2a10ea4d744d0e9a428914a56c6b7b3a3c5</t>
+        </is>
+      </c>
+      <c r="C229">
+        <v>32544</v>
+      </c>
+      <c r="D229">
+        <v>1280</v>
+      </c>
+      <c r="E229">
+        <v>900</v>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H229">
+        <v>0</v>
+      </c>
+      <c r="I229">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">438ee621fc826ae9fed1506da711bdfa22741878cecffcc74f55ddd47a9f5580</t>
+        </is>
+      </c>
+      <c r="C230">
+        <v>25539</v>
+      </c>
+      <c r="D230">
+        <v>390</v>
+      </c>
+      <c r="E230">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5dc4060a4fbfc7abf43eb94dd0b5510a94607a299559ede998822f6762ce8c26</t>
+        </is>
+      </c>
+      <c r="C231">
+        <v>25144</v>
+      </c>
+      <c r="D231">
+        <v>390</v>
+      </c>
+      <c r="E231">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1a092cf900b35c8ed127964ab62eee9d62a5f739f7cc66d1cb38593b8904544c</t>
+        </is>
+      </c>
+      <c r="C232">
+        <v>70165</v>
+      </c>
+      <c r="D232">
+        <v>1280</v>
+      </c>
+      <c r="E232">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">944a15f28baa2d26ba6016bd8004a545fe43dd3c35aa6ce372b107350d346eac</t>
+        </is>
+      </c>
+      <c r="C233">
+        <v>69288</v>
+      </c>
+      <c r="D233">
+        <v>1280</v>
+      </c>
+      <c r="E233">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">65d084d92fbb12be15d26ea1e667423f0fe879bab8470b842ffc5e1460fed6f3</t>
+        </is>
+      </c>
+      <c r="C234">
+        <v>35649</v>
+      </c>
+      <c r="D234">
+        <v>390</v>
+      </c>
+      <c r="E234">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">86927b021044a74874668f691445734d7d6233728ff23cbd05c5be6d5f385287</t>
+        </is>
+      </c>
+      <c r="C235">
+        <v>34690</v>
+      </c>
+      <c r="D235">
+        <v>390</v>
+      </c>
+      <c r="E235">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c8e90f15770799ed519cd8f248a7202dee1457066a166d53a407961e134de405</t>
+        </is>
+      </c>
+      <c r="C236">
+        <v>34641</v>
+      </c>
+      <c r="D236">
+        <v>390</v>
+      </c>
+      <c r="E236">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0afe486402d1cce5e2035ded1cc3627e90a90cf49557bc7fc73e4dfa55edf158</t>
+        </is>
+      </c>
+      <c r="C237">
+        <v>33682</v>
+      </c>
+      <c r="D237">
+        <v>390</v>
+      </c>
+      <c r="E237">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f951c018ce8a5e9090ae472ec51db8016e40089a2f622d36750a81797c2a29b0</t>
+        </is>
+      </c>
+      <c r="C238">
+        <v>78134</v>
+      </c>
+      <c r="D238">
+        <v>1280</v>
+      </c>
+      <c r="E238">
+        <v>900</v>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H238">
+        <v>15</v>
+      </c>
+      <c r="I238">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e835e862587ba313cd14842c289e719b5193e140ecb045afc966a205f4322cff</t>
+        </is>
+      </c>
+      <c r="C239">
+        <v>77276</v>
+      </c>
+      <c r="D239">
+        <v>1280</v>
+      </c>
+      <c r="E239">
+        <v>900</v>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H239">
+        <v>12</v>
+      </c>
+      <c r="I239">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">04f48d64ae27be0da886b91dcf517585ff3e42278c7ceca762c8bb5327c25798</t>
+        </is>
+      </c>
+      <c r="C240">
+        <v>43078</v>
+      </c>
+      <c r="D240">
+        <v>390</v>
+      </c>
+      <c r="E240">
+        <v>844</v>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H240">
+        <v>15</v>
+      </c>
+      <c r="I240">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d9a07d21d26651885f0b368001918215e76085466b9412df8a0e053b5d826523</t>
+        </is>
+      </c>
+      <c r="C241">
+        <v>42203</v>
+      </c>
+      <c r="D241">
+        <v>390</v>
+      </c>
+      <c r="E241">
+        <v>844</v>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H241">
+        <v>12</v>
+      </c>
+      <c r="I241">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I219"/>
+  <autoFilter ref="A1:I241"/>
 </worksheet>
 </file>
 
@@ -25867,12 +26534,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -25904,12 +26571,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -25941,12 +26608,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -25978,12 +26645,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -26015,12 +26682,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -26052,12 +26719,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -26089,12 +26756,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -26126,12 +26793,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -26163,12 +26830,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -26200,12 +26867,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -26237,12 +26904,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -26274,12 +26941,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -26311,12 +26978,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -26348,12 +27015,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -26385,12 +27052,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-empty-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-dark.png</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-dark.png</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -26422,12 +27089,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -26459,12 +27126,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -26496,12 +27163,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-10-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -26523,7 +27190,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="56" customWidth="1"/>
+    <col min="1" max="1" width="66" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
@@ -26558,7 +27225,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">599 tests/47files on final round8 source; /tmp/kynotes-affordance-r8-unit-final.log.</t>
+          <t xml:space="preserve">599 tests/47files on round9 source; /tmp/kynotes-alignment-r9-unit.log.</t>
         </is>
       </c>
     </row>
@@ -26575,7 +27242,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Final round8 TS/build/exact embed pass; /tmp/kynotes-affordance-r8-build-final.log. Existing603kBBlockNote warning.</t>
+          <t xml:space="preserve">Round9 TS/build/exact embed pass; /tmp/kynotes-alignment-r9-build.log. Existing603kB BlockNote warning.</t>
         </is>
       </c>
     </row>
@@ -26592,7 +27259,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/12 fresh-server browsers first attempt on final round8 source; /tmp/kynotes-affordance-r8-browser.log.</t>
+          <t xml:space="preserve">12/12 fresh-server browsers, first attempt on round9 source; /tmp/kynotes-alignment-r9-browser.log.</t>
         </is>
       </c>
     </row>
@@ -26660,7 +27327,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round8 staged tree9327c94f64ffac83b5354708726364bd1b4df09b; two private clean archives,CGO_ENABLED=0,-trimpath,release0.0.0. BothSHA2564edf95b5bafa4b324967ff8d9ae1db3079deb9f1f1105c1d147c8510186db176; /tmp/kynotes-affordance-r8-repeatability.log. Later evidence/AGENTS metadata cannot affect binary.</t>
+          <t xml:space="preserve">Round9 staged tree40eecf04a440cf0b9f550e106f2c9a5e1a0344; two private clean archives, CGO_ENABLED=0, -trimpath, release0.0.0. Both SHA256c3018f48866b7a677905836056bb13d66af31afe8b73a8a91a6b286e1e63d3ca.</t>
         </is>
       </c>
     </row>
@@ -26762,7 +27429,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current kynotes-affordance:r8 image,14step probe/setup pass; /tmp/kynotes-affordance-r8-{docker,probe,setup}.log.</t>
+          <t xml:space="preserve">Current kynotes-alignment:r9 image,14-step probe/setup pass; /tmp/kynotes-alignment-r9-{docker,probe,setup}.log.</t>
         </is>
       </c>
     </row>
@@ -26779,7 +27446,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round8 changed-source detector only existing semantic warning rail and overridden section-color border; affordance-round8-detector.json.</t>
+          <t xml:space="preserve">Round9 detector retains only existing semantic warning rail and overridden section-color border; alignment-round9-detector.json.</t>
         </is>
       </c>
     </row>
@@ -26953,8 +27620,25 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage12 control matching/phone alignment capture and regressions</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pass</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22captures/18unique, first attempt21.5s, fresh18112 fixture; /tmp/kynotes-alignment-r9-capture.log. Native390x844 body x17 versus title x16 (1px box border), padding16px0; desktop both plus controls40x40/radius8px with identical NavIcon paths and strong ink. No stored coordinates changed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C25"/>
+  <autoFilter ref="A1:C26"/>
 </worksheet>
 </file>
 
@@ -27021,7 +27705,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage11 after; all earlier inputs retained</t>
+          <t xml:space="preserve">Stage12 after; all earlier inputs retained</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: give phone settings evenly sized navigation
</commit_message>
<xml_diff>
--- a/docs/ui-notes-eight/KyNotes-Council.xlsx
+++ b/docs/ui-notes-eight/KyNotes-Council.xlsx
@@ -444,8 +444,53 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deferred</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate raw verdicts; Gemini raw* is excluded from progression because its weights/claims fail the audit. See original reviews and Gemini audit.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not scored</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I11"/>
 </worksheet>
 </file>
 
@@ -29478,8 +29523,662 @@
         <v>4</v>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c75e0f370c7b318a30b96856e857ddee878c559633886009ce2f34bb8916cc89</t>
+        </is>
+      </c>
+      <c r="C242">
+        <v>69755</v>
+      </c>
+      <c r="D242">
+        <v>1280</v>
+      </c>
+      <c r="E242">
+        <v>900</v>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H242">
+        <v>0</v>
+      </c>
+      <c r="I242">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1e65157f29c09998407a3643285cd11506950fc1784b9e24c48f27a5bc98e1fe</t>
+        </is>
+      </c>
+      <c r="C243">
+        <v>68773</v>
+      </c>
+      <c r="D243">
+        <v>1280</v>
+      </c>
+      <c r="E243">
+        <v>900</v>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-appearance-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H243">
+        <v>0</v>
+      </c>
+      <c r="I243">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f77379a3fcef8de6ad3a2debef934f700605e9b398ca1d2268bf0bf89dc6c15b</t>
+        </is>
+      </c>
+      <c r="C244">
+        <v>40691</v>
+      </c>
+      <c r="D244">
+        <v>390</v>
+      </c>
+      <c r="E244">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43accf28ed4061ec3747d6df7aca86e11f15813cb78f27d1511f8a979bfb9488</t>
+        </is>
+      </c>
+      <c r="C245">
+        <v>40096</v>
+      </c>
+      <c r="D245">
+        <v>390</v>
+      </c>
+      <c r="E245">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e1585cc65bdba3dcd62c8c4caed04471c64dbf25395a24283025fb3459d6b568</t>
+        </is>
+      </c>
+      <c r="C246">
+        <v>78102</v>
+      </c>
+      <c r="D246">
+        <v>1280</v>
+      </c>
+      <c r="E246">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ff94b5e57447ea81cb8346ffc28e9bd80002715029499914b3bc9611027c6154</t>
+        </is>
+      </c>
+      <c r="C247">
+        <v>77310</v>
+      </c>
+      <c r="D247">
+        <v>1280</v>
+      </c>
+      <c r="E247">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2fb0e5a699ffb0d4f8987c771973343b7ea20db1f97b67550de6a244a1711317</t>
+        </is>
+      </c>
+      <c r="C248">
+        <v>43038</v>
+      </c>
+      <c r="D248">
+        <v>390</v>
+      </c>
+      <c r="E248">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">992939e77969e7265590263e5632fe52c48d71a191d60efadcc1baefeebc9721</t>
+        </is>
+      </c>
+      <c r="C249">
+        <v>42235</v>
+      </c>
+      <c r="D249">
+        <v>390</v>
+      </c>
+      <c r="E249">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6bb7c1e9f1bb2e595fef91ad00eb7b483b20fdf7832825094759ef38fc277b1a</t>
+        </is>
+      </c>
+      <c r="C250">
+        <v>32909</v>
+      </c>
+      <c r="D250">
+        <v>1280</v>
+      </c>
+      <c r="E250">
+        <v>900</v>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H250">
+        <v>0</v>
+      </c>
+      <c r="I250">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">70340422c86d96f05b2de950ae87c2a10ea4d744d0e9a428914a56c6b7b3a3c5</t>
+        </is>
+      </c>
+      <c r="C251">
+        <v>32544</v>
+      </c>
+      <c r="D251">
+        <v>1280</v>
+      </c>
+      <c r="E251">
+        <v>900</v>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-10-after-empty-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H251">
+        <v>0</v>
+      </c>
+      <c r="I251">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">438ee621fc826ae9fed1506da711bdfa22741878cecffcc74f55ddd47a9f5580</t>
+        </is>
+      </c>
+      <c r="C252">
+        <v>25539</v>
+      </c>
+      <c r="D252">
+        <v>390</v>
+      </c>
+      <c r="E252">
+        <v>844</v>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H252">
+        <v>0</v>
+      </c>
+      <c r="I252">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5dc4060a4fbfc7abf43eb94dd0b5510a94607a299559ede998822f6762ce8c26</t>
+        </is>
+      </c>
+      <c r="C253">
+        <v>25144</v>
+      </c>
+      <c r="D253">
+        <v>390</v>
+      </c>
+      <c r="E253">
+        <v>844</v>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H253">
+        <v>0</v>
+      </c>
+      <c r="I253">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a75b5d14d72ca58a593433a739dac278c43df8110168d8e3e9618590e9cf2d67</t>
+        </is>
+      </c>
+      <c r="C254">
+        <v>70149</v>
+      </c>
+      <c r="D254">
+        <v>1280</v>
+      </c>
+      <c r="E254">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0d7bd1d2401656ebebe6550adefb48507a123b5f996031ae853bec7e6ccad552</t>
+        </is>
+      </c>
+      <c r="C255">
+        <v>69312</v>
+      </c>
+      <c r="D255">
+        <v>1280</v>
+      </c>
+      <c r="E255">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">330ad34a5ab0520cfe46ac9997414e78c1c37ef2ba660f2a1890afa3af3118e9</t>
+        </is>
+      </c>
+      <c r="C256">
+        <v>35610</v>
+      </c>
+      <c r="D256">
+        <v>390</v>
+      </c>
+      <c r="E256">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">134934efa19faf305471030860f78badf166b8bfb4a93cd3d0f6e7e9510b4bb8</t>
+        </is>
+      </c>
+      <c r="C257">
+        <v>34717</v>
+      </c>
+      <c r="D257">
+        <v>390</v>
+      </c>
+      <c r="E257">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c8e90f15770799ed519cd8f248a7202dee1457066a166d53a407961e134de405</t>
+        </is>
+      </c>
+      <c r="C258">
+        <v>34641</v>
+      </c>
+      <c r="D258">
+        <v>390</v>
+      </c>
+      <c r="E258">
+        <v>844</v>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H258">
+        <v>0</v>
+      </c>
+      <c r="I258">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0afe486402d1cce5e2035ded1cc3627e90a90cf49557bc7fc73e4dfa55edf158</t>
+        </is>
+      </c>
+      <c r="C259">
+        <v>33682</v>
+      </c>
+      <c r="D259">
+        <v>390</v>
+      </c>
+      <c r="E259">
+        <v>844</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact</t>
+        </is>
+      </c>
+      <c r="H259">
+        <v>0</v>
+      </c>
+      <c r="I259">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-workspace-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aa2d4ff1bf002592b3e57a060fd369f0616441672db8834aaa3038be5d7f055c</t>
+        </is>
+      </c>
+      <c r="C260">
+        <v>78103</v>
+      </c>
+      <c r="D260">
+        <v>1280</v>
+      </c>
+      <c r="E260">
+        <v>900</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-desktop-dark.png</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H260">
+        <v>15</v>
+      </c>
+      <c r="I260">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-workspace-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">092436455f3088abd4a444fbb7138baeb1aeb17139401955f4cd9a264587ccbd</t>
+        </is>
+      </c>
+      <c r="C261">
+        <v>77304</v>
+      </c>
+      <c r="D261">
+        <v>1280</v>
+      </c>
+      <c r="E261">
+        <v>900</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-desktop-light.png</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H261">
+        <v>12</v>
+      </c>
+      <c r="I261">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-workspace-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3d0e83693140945cf96e89c89a6dfc07779acfc3dcd10bec4aebbda54f9abb06</t>
+        </is>
+      </c>
+      <c r="C262">
+        <v>43040</v>
+      </c>
+      <c r="D262">
+        <v>390</v>
+      </c>
+      <c r="E262">
+        <v>844</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-mobile-dark.png</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H262">
+        <v>15</v>
+      </c>
+      <c r="I262">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-workspace-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fac0ca1bed8abb9f5444ed5e84c4886f1cf40a3ad44d332eb32b4088633fb71a</t>
+        </is>
+      </c>
+      <c r="C263">
+        <v>42227</v>
+      </c>
+      <c r="D263">
+        <v>390</v>
+      </c>
+      <c r="E263">
+        <v>844</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-mobile-light.png</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">near (rasterization; measured bounds recorded)</t>
+        </is>
+      </c>
+      <c r="H263">
+        <v>12</v>
+      </c>
+      <c r="I263">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I241"/>
+  <autoFilter ref="A1:I263"/>
 </worksheet>
 </file>
 
@@ -29550,12 +30249,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-desktop-light.png</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -29587,12 +30286,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-desktop-light.png</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -29624,12 +30323,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-desktop-light.png</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -29661,12 +30360,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-desktop-light.png</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -29698,12 +30397,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-editor-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-desktop-dark.png</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -29735,12 +30434,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-empty-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-desktop-dark.png</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -29772,12 +30471,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-desktop-dark.png</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -29809,12 +30508,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-desktop-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-desktop-dark.png</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -29846,12 +30545,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-mobile-light.png</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -29883,12 +30582,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-mobile-light.png</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -29920,12 +30619,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-mobile-light.png</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -29957,12 +30656,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-pages-mobile-light.png</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -29994,12 +30693,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-light.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-mobile-light.png</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -30031,12 +30730,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-editor-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-editor-mobile-dark.png</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -30068,12 +30767,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-empty-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-dark.png</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-empty-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-empty-mobile-dark.png</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -30105,12 +30804,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-appearance-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-appearance-mobile-dark.png</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -30142,12 +30841,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-pages-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-pages-mobile-dark.png</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -30179,12 +30878,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-11-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">screenshots/kynotes-12-after-navigation-mobile-dark.png</t>
+          <t xml:space="preserve">screenshots/kynotes-13-after-navigation-mobile-dark.png</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -30241,7 +30940,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">599 tests/47files on round9 source; /tmp/kynotes-alignment-r9-unit.log.</t>
+          <t xml:space="preserve">599 tests/47files on round10 source; /tmp/kynotes-settings-r10-unit.log.</t>
         </is>
       </c>
     </row>
@@ -30258,7 +30957,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round9 TS/build/exact embed pass; /tmp/kynotes-alignment-r9-build.log. Existing603kB BlockNote warning.</t>
+          <t xml:space="preserve">Round10 TS/build/exact embed pass; /tmp/kynotes-settings-r10-build.log. Existing603kB BlockNote warning.</t>
         </is>
       </c>
     </row>
@@ -30275,7 +30974,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/12 fresh-server browsers, first attempt on round9 source; /tmp/kynotes-alignment-r9-browser.log.</t>
+          <t xml:space="preserve">12/12 fresh-server browsers, first attempt on round10 source; /tmp/kynotes-settings-r10-browser.log.</t>
         </is>
       </c>
     </row>
@@ -30343,7 +31042,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round9 staged tree40eecf04a440cf0b9f550e106f2c9a945e1a0344; two private clean archives, CGO_ENABLED=0, -trimpath, release0.0.0. Both SHA256c3018f48866b7a677905836056bb13d66af31afe8b73a8a91a6b286e1e63d3ca.</t>
+          <t xml:space="preserve">Round10 staged tree155ee40d5d9ccedc0038983531b5baed9c0750da; two private clean archives, CGO_ENABLED=0, -trimpath, release0.0.0. Both SHA25671a7029b823f70e8e1e835c7f4feff5b3140435acef4ff5809af855753f6ff1c; /tmp/kynotes-settings-r10-repeatability.log.</t>
         </is>
       </c>
     </row>
@@ -30445,7 +31144,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current kynotes-alignment:r9 image,14-step probe/setup pass; /tmp/kynotes-alignment-r9-{docker,probe,setup}.log.</t>
+          <t xml:space="preserve">Current kynotes-settings:r10 image,14-step probe/setup pass; /tmp/kynotes-settings-r10-{docker,probe,setup}.log.</t>
         </is>
       </c>
     </row>
@@ -30462,7 +31161,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Round9 detector retains only existing semantic warning rail and overridden section-color border; alignment-round9-detector.json.</t>
+          <t xml:space="preserve">Round10 detector retains only existing semantic warning rail and overridden section-color border; settings-round10-detector.json.</t>
         </is>
       </c>
     </row>
@@ -30653,8 +31352,42 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage13 phone Settings layout capture and regressions</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pass</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22captures/18unique, first attempt26.3s, fresh18114 fixture; /tmp/kynotes-settings-r10-capture.log. Native390light/dark two40px link rows, all6anchors resolve,23radios,no savedchoice and Appearance44px higher.800/1280also overflow0;320baseline15pxoverflow retained and separately recorded in theme-checks/round10-native-settings.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Historical inventory correction</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pass</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inventory-v12 unions10 missed exactSHA groups, removing24 excess representatives without changing any image or score. Corrected stage12:240PNGs/184SHA groups/138normalized groups. Stage13 inventory-v13:262PNGs/148normalized groups; no duplicate chains or false exact links. round9-evidence-audit.json corrects Opus exact-versus-normalized wording and parent repeatability tree typo.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C26"/>
+  <autoFilter ref="A1:C28"/>
 </worksheet>
 </file>
 
@@ -30721,7 +31454,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage12 after; all earlier inputs retained</t>
+          <t xml:space="preserve">Stage13 after; all earlier inputs retained</t>
         </is>
       </c>
     </row>

</xml_diff>